<commit_message>
Initial commit - Mini ERP application
</commit_message>
<xml_diff>
--- a/data/Sources.xlsx
+++ b/data/Sources.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pfnonwovens-my.sharepoint.com/personal/mfischer_pfnonwovens_com/Documents/Desktop/mini-erp-node/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="8_{66A118C3-EF46-4704-A6DB-C24509B266D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC1485AA-200A-4634-89A8-B41967906580}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="8_{66A118C3-EF46-4704-A6DB-C24509B266D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF32266F-029E-4EC8-8A76-FC6A52D9D36D}"/>
   <bookViews>
-    <workbookView xWindow="28425" yWindow="-10335" windowWidth="30570" windowHeight="17070" xr2:uid="{B924FA10-533B-4C07-A917-FCB6B882FB42}"/>
+    <workbookView xWindow="34320" yWindow="21600" windowWidth="17415" windowHeight="20985" xr2:uid="{B924FA10-533B-4C07-A917-FCB6B882FB42}"/>
   </bookViews>
   <sheets>
     <sheet name="Lists" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="445">
   <si>
     <t>SB1</t>
   </si>
@@ -1347,6 +1347,42 @@
   </si>
   <si>
     <t>Pig - M-Color šedý 80 620 PP-2</t>
+  </si>
+  <si>
+    <t>5800 eC/S</t>
+  </si>
+  <si>
+    <t>6800 C/S</t>
+  </si>
+  <si>
+    <t>6800 S/S</t>
+  </si>
+  <si>
+    <t>2500 C/S 0,55</t>
+  </si>
+  <si>
+    <t>2500 C/S 0,65</t>
+  </si>
+  <si>
+    <t>eC/S 5800+S/S 6800</t>
+  </si>
+  <si>
+    <t>6800 C/S (+ blocking plate =total 4800cpm; c=0,55mm)</t>
+  </si>
+  <si>
+    <t>2500 C/S + 1100 C/S</t>
+  </si>
+  <si>
+    <t>S/S 5800+S/S 6800</t>
+  </si>
+  <si>
+    <t>trilobal C/S</t>
+  </si>
+  <si>
+    <t>eC/S 5800 + C/S 1100</t>
+  </si>
+  <si>
+    <t>eC/S 5800</t>
   </si>
 </sst>
 </file>
@@ -1709,7 +1745,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1899,20 +1935,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="4" fontId="10" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="10" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1931,8 +1953,21 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="4" fontId="10" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="10" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3484,7 +3519,7 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
+    <xxl21:alternateUrls driveId="b!CD23Tkh7ckaGyHyK3EY_0B_jrMQaaRZOgvj_ynpV64SFnLEixdoOS4nwLSg-q2ic" itemId="01RPP366CMSLVINGTTMREZCHFIYNMR6IUT">
       <xxl21:absoluteUrl r:id="rId2"/>
     </xxl21:alternateUrls>
     <sheetNames>
@@ -3529,8 +3564,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{4905E39C-E898-4DCE-8992-EB9DD8BDD77C}" name="Structure" displayName="Structure" ref="K1:K5" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36" headerRowCellStyle="Normální 2">
-  <autoFilter ref="K1:K5" xr:uid="{4905E39C-E898-4DCE-8992-EB9DD8BDD77C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{4905E39C-E898-4DCE-8992-EB9DD8BDD77C}" name="Structure" displayName="Structure" ref="K1:K17" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36" headerRowCellStyle="Normální 2">
+  <autoFilter ref="K1:K17" xr:uid="{4905E39C-E898-4DCE-8992-EB9DD8BDD77C}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{56A23D9B-6A6F-4753-BE1E-C32EC840E0CC}" name="Structure" dataDxfId="35"/>
   </tableColumns>
@@ -4143,7 +4178,7 @@
       <c r="M2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="N2" s="69" t="s">
+      <c r="N2" s="7" t="s">
         <v>277</v>
       </c>
       <c r="O2" s="7" t="s">
@@ -4364,6 +4399,9 @@
       <c r="I6" s="5" t="s">
         <v>61</v>
       </c>
+      <c r="K6" s="68" t="s">
+        <v>433</v>
+      </c>
       <c r="L6" s="7" t="s">
         <v>62</v>
       </c>
@@ -4411,8 +4449,11 @@
       <c r="G7" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="H7" s="68" t="s">
+      <c r="H7" s="5" t="s">
         <v>277</v>
+      </c>
+      <c r="K7" s="68" t="s">
+        <v>434</v>
       </c>
       <c r="L7" s="7" t="s">
         <v>71</v>
@@ -4455,6 +4496,9 @@
       <c r="G8" s="5" t="s">
         <v>78</v>
       </c>
+      <c r="K8" s="68" t="s">
+        <v>435</v>
+      </c>
       <c r="L8" s="7" t="s">
         <v>79</v>
       </c>
@@ -4496,6 +4540,9 @@
       <c r="G9" s="5" t="s">
         <v>85</v>
       </c>
+      <c r="K9" s="68" t="s">
+        <v>436</v>
+      </c>
       <c r="L9" s="7" t="s">
         <v>86</v>
       </c>
@@ -4537,6 +4584,9 @@
       <c r="G10" s="5" t="s">
         <v>92</v>
       </c>
+      <c r="K10" s="68" t="s">
+        <v>437</v>
+      </c>
       <c r="L10" s="7" t="s">
         <v>93</v>
       </c>
@@ -4578,6 +4628,9 @@
       <c r="G11" s="5" t="s">
         <v>99</v>
       </c>
+      <c r="K11" s="68" t="s">
+        <v>438</v>
+      </c>
       <c r="L11" s="7" t="s">
         <v>100</v>
       </c>
@@ -4619,6 +4672,9 @@
       <c r="G12" s="5" t="s">
         <v>105</v>
       </c>
+      <c r="K12" s="68" t="s">
+        <v>439</v>
+      </c>
       <c r="L12" s="7" t="s">
         <v>106</v>
       </c>
@@ -4657,6 +4713,9 @@
       <c r="G13" s="5" t="s">
         <v>112</v>
       </c>
+      <c r="K13" s="68" t="s">
+        <v>440</v>
+      </c>
       <c r="L13" s="7" t="s">
         <v>113</v>
       </c>
@@ -4695,6 +4754,9 @@
       <c r="G14" s="5" t="s">
         <v>119</v>
       </c>
+      <c r="K14" s="68" t="s">
+        <v>441</v>
+      </c>
       <c r="L14" s="7" t="s">
         <v>120</v>
       </c>
@@ -4730,6 +4792,9 @@
       <c r="G15" s="5" t="s">
         <v>125</v>
       </c>
+      <c r="K15" s="68" t="s">
+        <v>442</v>
+      </c>
       <c r="L15" s="7" t="s">
         <v>126</v>
       </c>
@@ -4760,6 +4825,9 @@
       <c r="G16" s="5" t="s">
         <v>129</v>
       </c>
+      <c r="K16" s="68" t="s">
+        <v>443</v>
+      </c>
       <c r="L16" s="7" t="s">
         <v>130</v>
       </c>
@@ -4789,6 +4857,9 @@
       </c>
       <c r="G17" s="5" t="s">
         <v>133</v>
+      </c>
+      <c r="K17" s="68" t="s">
+        <v>444</v>
       </c>
       <c r="L17" s="7" t="s">
         <v>134</v>
@@ -5850,14 +5921,14 @@
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" s="10"/>
       <c r="B3" s="10"/>
-      <c r="C3" s="62" t="s">
+      <c r="C3" s="58" t="s">
         <v>269</v>
       </c>
-      <c r="D3" s="63"/>
-      <c r="E3" s="62" t="s">
+      <c r="D3" s="59"/>
+      <c r="E3" s="58" t="s">
         <v>269</v>
       </c>
-      <c r="F3" s="63"/>
+      <c r="F3" s="59"/>
       <c r="G3" s="14" t="s">
         <v>13</v>
       </c>
@@ -5870,14 +5941,14 @@
       <c r="J3" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="K3" s="64" t="s">
+      <c r="K3" s="60" t="s">
         <v>269</v>
       </c>
-      <c r="L3" s="65"/>
-      <c r="M3" s="62" t="s">
+      <c r="L3" s="61"/>
+      <c r="M3" s="58" t="s">
         <v>269</v>
       </c>
-      <c r="N3" s="63"/>
+      <c r="N3" s="59"/>
       <c r="O3" s="9"/>
       <c r="P3" s="9"/>
       <c r="Q3" s="13"/>
@@ -5897,14 +5968,14 @@
         <v>396</v>
       </c>
       <c r="B4" s="16"/>
-      <c r="C4" s="66" t="s">
+      <c r="C4" s="62" t="s">
         <v>397</v>
       </c>
-      <c r="D4" s="67"/>
-      <c r="E4" s="66" t="s">
+      <c r="D4" s="63"/>
+      <c r="E4" s="62" t="s">
         <v>398</v>
       </c>
-      <c r="F4" s="67"/>
+      <c r="F4" s="63"/>
       <c r="G4" s="17" t="s">
         <v>399</v>
       </c>
@@ -5917,14 +5988,14 @@
       <c r="J4" s="15" t="s">
         <v>402</v>
       </c>
-      <c r="K4" s="66" t="s">
+      <c r="K4" s="62" t="s">
         <v>403</v>
       </c>
-      <c r="L4" s="67"/>
-      <c r="M4" s="66" t="s">
+      <c r="L4" s="63"/>
+      <c r="M4" s="62" t="s">
         <v>404</v>
       </c>
-      <c r="N4" s="67"/>
+      <c r="N4" s="63"/>
       <c r="O4" s="9"/>
       <c r="P4" s="9"/>
       <c r="Q4" s="9"/>
@@ -5944,22 +6015,22 @@
         <v>405</v>
       </c>
       <c r="B5" s="18"/>
-      <c r="C5" s="58">
+      <c r="C5" s="64">
         <v>34.700000000000003</v>
       </c>
-      <c r="D5" s="59"/>
-      <c r="E5" s="58"/>
-      <c r="F5" s="59"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="65"/>
       <c r="G5" s="19">
         <v>5.3</v>
       </c>
       <c r="H5" s="20"/>
       <c r="I5" s="19"/>
       <c r="J5" s="19"/>
-      <c r="K5" s="58"/>
-      <c r="L5" s="59"/>
-      <c r="M5" s="58"/>
-      <c r="N5" s="59"/>
+      <c r="K5" s="64"/>
+      <c r="L5" s="65"/>
+      <c r="M5" s="64"/>
+      <c r="N5" s="65"/>
       <c r="O5" s="21">
         <f>SUM(C5:N5)</f>
         <v>40</v>
@@ -5982,16 +6053,16 @@
         <v>406</v>
       </c>
       <c r="B6" s="25"/>
-      <c r="C6" s="60">
+      <c r="C6" s="66">
         <f>C5/$O$5</f>
         <v>0.86750000000000005</v>
       </c>
-      <c r="D6" s="61"/>
-      <c r="E6" s="60">
+      <c r="D6" s="67"/>
+      <c r="E6" s="66">
         <f>E5/$O$5</f>
         <v>0</v>
       </c>
-      <c r="F6" s="61"/>
+      <c r="F6" s="67"/>
       <c r="G6" s="26">
         <f>G5/$O$5</f>
         <v>0.13250000000000001</v>
@@ -6008,16 +6079,16 @@
         <f>J5/$O$5</f>
         <v>0</v>
       </c>
-      <c r="K6" s="60">
+      <c r="K6" s="66">
         <f>K5/$O$5</f>
         <v>0</v>
       </c>
-      <c r="L6" s="61"/>
-      <c r="M6" s="60">
+      <c r="L6" s="67"/>
+      <c r="M6" s="66">
         <f>M5/$O$5</f>
         <v>0</v>
       </c>
-      <c r="N6" s="61"/>
+      <c r="N6" s="67"/>
       <c r="O6" s="27">
         <f>SUM(C6:N6)</f>
         <v>1</v>
@@ -7017,6 +7088,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="M5:N5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="M6:N6"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="K3:L3"/>
@@ -7025,14 +7104,6 @@
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="K4:L4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="M5:N5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="M6:N6"/>
   </mergeCells>
   <conditionalFormatting sqref="A29">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="notEqual">

</xml_diff>

<commit_message>
BOM Calculation page adjustments
</commit_message>
<xml_diff>
--- a/data/Sources.xlsx
+++ b/data/Sources.xlsx
@@ -2,23 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pfnonwovens-my.sharepoint.com/personal/mfischer_pfnonwovens_com/Documents/Desktop/mini-erp-node/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="65" documentId="8_{66A118C3-EF46-4704-A6DB-C24509B266D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0ECF8CCB-948B-44AE-922D-560B6C578378}"/>
+  <xr:revisionPtr revIDLastSave="79" documentId="8_{66A118C3-EF46-4704-A6DB-C24509B266D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37174538-E850-4CAF-AE52-6F19ADE6659F}"/>
   <bookViews>
-    <workbookView xWindow="33555" yWindow="-9315" windowWidth="21600" windowHeight="12585" xr2:uid="{B924FA10-533B-4C07-A917-FCB6B882FB42}"/>
+    <workbookView xWindow="30105" yWindow="-7095" windowWidth="22575" windowHeight="12585" activeTab="2" xr2:uid="{B924FA10-533B-4C07-A917-FCB6B882FB42}"/>
   </bookViews>
   <sheets>
     <sheet name="Lists" sheetId="1" r:id="rId1"/>
     <sheet name="Calc" sheetId="2" r:id="rId2"/>
+    <sheet name="TechParams" sheetId="3" r:id="rId3"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId3"/>
-  </externalReferences>
   <definedNames>
     <definedName name="list_additive">Additive[Additive]</definedName>
     <definedName name="list_mb">MB[MB]</definedName>
@@ -47,8 +45,44 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>KPokorny</author>
+  </authors>
+  <commentList>
+    <comment ref="Y9" authorId="0" shapeId="0" xr:uid="{E14AD1C4-87B7-4202-B01A-EC18338EA8FE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="238"/>
+          </rPr>
+          <t>KPokorny:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="238"/>
+          </rPr>
+          <t xml:space="preserve">
+100mm je odhad. Nebylo testováno po výměně krytů na předních nožích.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="548">
   <si>
     <t>SB1</t>
   </si>
@@ -164,9 +198,6 @@
     <t>hygiene</t>
   </si>
   <si>
-    <t>SM</t>
-  </si>
-  <si>
     <t>Mono</t>
   </si>
   <si>
@@ -200,9 +231,6 @@
     <t>medical</t>
   </si>
   <si>
-    <t>SMM</t>
-  </si>
-  <si>
     <t>SS</t>
   </si>
   <si>
@@ -1401,6 +1429,327 @@
   </si>
   <si>
     <t>090/10</t>
+  </si>
+  <si>
+    <t>CZ12s (200%)</t>
+  </si>
+  <si>
+    <t>CZ12b (150%)</t>
+  </si>
+  <si>
+    <t>CZ12a (180%)</t>
+  </si>
+  <si>
+    <t>Linka</t>
+  </si>
+  <si>
+    <t>Konfigurace</t>
+  </si>
+  <si>
+    <t>Šířka trysek    (m)</t>
+  </si>
+  <si>
+    <t>Šířka sítového pásu                 ( m )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Využitelná šířka NT        **                                                                                                                                                          min / max                                                                                    </t>
+  </si>
+  <si>
+    <t>Min. rychlost pásu / max. gsm</t>
+  </si>
+  <si>
+    <t>Max. rychlost pásu / min. gsm</t>
+  </si>
+  <si>
+    <t>Min. výkon SB hlavy                 kg/h/m</t>
+  </si>
+  <si>
+    <t>Optimální výkon SB kg/h/m</t>
+  </si>
+  <si>
+    <t>Max. výkon SB hlavy   kg/h/m</t>
+  </si>
+  <si>
+    <t>Min. výkon MB hlavy    kg/h/m</t>
+  </si>
+  <si>
+    <t>Optimální výkon MB hlavy    kg/h/m</t>
+  </si>
+  <si>
+    <t>Max. výkon MB hlavy        kg/h/m</t>
+  </si>
+  <si>
+    <t>Max. počet nožů</t>
+  </si>
+  <si>
+    <t>Min. šířka nožů           ( mm )</t>
+  </si>
+  <si>
+    <t>Mono G1</t>
+  </si>
+  <si>
+    <t>Mono G2</t>
+  </si>
+  <si>
+    <t>Mono G3 / G6</t>
+  </si>
+  <si>
+    <t>SMS G1</t>
+  </si>
+  <si>
+    <t>SMS G2</t>
+  </si>
+  <si>
+    <t>Bico G1</t>
+  </si>
+  <si>
+    <t>Bico G4 / G5</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>L01</t>
+  </si>
+  <si>
+    <t>10gsm 3,10m  130gsm 3,2m</t>
+  </si>
+  <si>
+    <t>14m/min.  130gsm</t>
+  </si>
+  <si>
+    <t>120m/min.  10gsm</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">60 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color indexed="60"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>(60mmrole)</t>
+    </r>
+  </si>
+  <si>
+    <t>L02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12gsm 3,05 m 100gsm 3,20 m </t>
+  </si>
+  <si>
+    <t>14,5gsm 3,2m    100gsm 3,2m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40m/min 100gsm </t>
+  </si>
+  <si>
+    <t>270m/min 10gsm</t>
+  </si>
+  <si>
+    <t>75 (70mmrole)</t>
+  </si>
+  <si>
+    <t>L03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10gsm 2,90m            80gsm 3,20m </t>
+  </si>
+  <si>
+    <t>15gsm 2,7m                25gsm 2,8m</t>
+  </si>
+  <si>
+    <t>15,6gsm 3,2m    55gsm 3,2m</t>
+  </si>
+  <si>
+    <t>45m/min 80gsm</t>
+  </si>
+  <si>
+    <t>450m/min 10gsm</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">75 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color indexed="60"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>(70mmrole)</t>
+    </r>
+  </si>
+  <si>
+    <t>L05</t>
+  </si>
+  <si>
+    <t>SSMMS</t>
+  </si>
+  <si>
+    <t>15gsm 2,860m          50gsm 3,276m</t>
+  </si>
+  <si>
+    <t>15gsm 3,1m</t>
+  </si>
+  <si>
+    <t>14gsm 2,90m       30gsm 3,1m</t>
+  </si>
+  <si>
+    <t>25gsm                2,646 / 2,688 m</t>
+  </si>
+  <si>
+    <t>159m/min           50gsm</t>
+  </si>
+  <si>
+    <t>580m/min          12gsm</t>
+  </si>
+  <si>
+    <t>L07</t>
+  </si>
+  <si>
+    <t>SSS</t>
+  </si>
+  <si>
+    <t>23gsm 3,180m   15gsm 2,945m</t>
+  </si>
+  <si>
+    <t>30gsm 3,080m   15gsm 2,656m</t>
+  </si>
+  <si>
+    <t>15gsm 3,16m  12gsm 2,730m</t>
+  </si>
+  <si>
+    <t>25gsm 2,856m  20gsm 2,652m</t>
+  </si>
+  <si>
+    <t>80m/min 80gsm</t>
+  </si>
+  <si>
+    <t>580 m/min 12gsm</t>
+  </si>
+  <si>
+    <t>L08</t>
+  </si>
+  <si>
+    <t>12gsm - 3,696    25gsm - 4,060</t>
+  </si>
+  <si>
+    <t>17gsm - 3,650 35gsm - 3,920</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13gsm G3-3,546 22gsm G6 3,876 </t>
+  </si>
+  <si>
+    <t>235m/min     50gsm</t>
+  </si>
+  <si>
+    <t>755m/min            12gsm</t>
+  </si>
+  <si>
+    <t>L09</t>
+  </si>
+  <si>
+    <t>SSMMMS</t>
+  </si>
+  <si>
+    <t>15gsm S-blend 2,800m</t>
+  </si>
+  <si>
+    <t>17gsm 2,900m</t>
+  </si>
+  <si>
+    <t>60gsm 3,100m   8gsm 2,880m</t>
+  </si>
+  <si>
+    <t>17gsm 2,975m</t>
+  </si>
+  <si>
+    <t>170m/min 60gsm</t>
+  </si>
+  <si>
+    <t>1000m/min 8gsm</t>
+  </si>
+  <si>
+    <t>37 (35funkčních)</t>
+  </si>
+  <si>
+    <t>L10</t>
+  </si>
+  <si>
+    <t>12gsm 4,100m   40g 4,300m</t>
+  </si>
+  <si>
+    <t>8gsm 4,000m    15gsm 4,312m</t>
+  </si>
+  <si>
+    <t>17gsm 4,180m</t>
+  </si>
+  <si>
+    <t>35gsm 4,136m</t>
+  </si>
+  <si>
+    <t>1150m/min   7gsm</t>
+  </si>
+  <si>
+    <t>EL01</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 25gsm  4,080m       12gsm 3,642m</t>
+  </si>
+  <si>
+    <t>22gsm 3,876m    13gsm 3,392m</t>
+  </si>
+  <si>
+    <t>15gsm 4,004m   10gsm 3,836m</t>
+  </si>
+  <si>
+    <t>L11</t>
+  </si>
+  <si>
+    <t>SMMS</t>
+  </si>
+  <si>
+    <t>40gsm 2,730m 12gsm 2,450m</t>
+  </si>
+  <si>
+    <t>20gsm 2,530m 8gsm 2,250m</t>
+  </si>
+  <si>
+    <t>17gsm 2,600</t>
+  </si>
+  <si>
+    <t>110m/min 60gsm</t>
+  </si>
+  <si>
+    <t>600m/min 8gsm</t>
+  </si>
+  <si>
+    <t>L12*</t>
+  </si>
+  <si>
+    <t>7gsm 2,160m</t>
+  </si>
+  <si>
+    <t>130m/min 60gsm</t>
+  </si>
+  <si>
+    <t>800 m/min</t>
+  </si>
+  <si>
+    <t>PET - 320 BICO - 240</t>
+  </si>
+  <si>
+    <t>** uvedená využitelná šířka je uvedena z komerční výroby a tyto čísla je nutno brát s rezervou, protože záleží na mnoha faktorech -  počet rolí, poměr PP/PE, množství MB v SMS….</t>
+  </si>
+  <si>
+    <t>* u této linky je HAK a HAF kde proudí horký vzduch kolem 150 - 170 °C</t>
   </si>
 </sst>
 </file>
@@ -1412,7 +1761,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1510,8 +1859,57 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="60"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1536,8 +1934,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="15"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="21">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -1771,12 +2181,91 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="1">
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal style="thin">
+        <color indexed="64"/>
+      </diagonal>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1967,19 +2456,58 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="10" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="21" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="10" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="21" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1999,12 +2527,28 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="4" fontId="10" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="10" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normální 2" xfId="1" xr:uid="{F0199B67-A81D-4A98-8F3A-51A8A4957AF3}"/>
+    <cellStyle name="Normální 4" xfId="2" xr:uid="{F16BADC3-D42A-4BE6-ADE9-7B86357C48FD}"/>
   </cellStyles>
   <dxfs count="68">
     <dxf>
@@ -3549,43 +4093,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls driveId="b!CD23Tkh7ckaGyHyK3EY_0B_jrMQaaRZOgvj_ynpV64SFnLEixdoOS4nwLSg-q2ic" itemId="01RPP366CMSLVINGTTMREZCHFIYNMR6IUT">
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Link to Old"/>
-      <sheetName val="Technické údaje linek (2)"/>
-      <sheetName val="Seznamy"/>
-      <sheetName val="Recyklace, regranulace"/>
-      <sheetName val="Základní informace"/>
-      <sheetName val="PP"/>
-      <sheetName val="Suroviny"/>
-      <sheetName val="PFN_EMEA_patterns"/>
-      <sheetName val="Odpady"/>
-      <sheetName val="Parametry linek"/>
-    </sheetNames>
-    <definedNames>
-      <definedName name="výmaz"/>
-    </definedNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FD2F10F3-78D8-42BB-8A3B-AA944E100804}" name="SB" displayName="SB" ref="A1:A31" totalsRowShown="0" headerRowDxfId="67" dataDxfId="65" headerRowBorderDxfId="66" tableBorderDxfId="64" headerRowCellStyle="Normální 2">
   <autoFilter ref="A1:A31" xr:uid="{FD2F10F3-78D8-42BB-8A3B-AA944E100804}"/>
@@ -3673,8 +4180,8 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{838775E4-F5E0-431D-9351-D17AE56F19D7}" name="Line" displayName="Line" ref="R1:R14" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
-  <autoFilter ref="R1:R14" xr:uid="{838775E4-F5E0-431D-9351-D17AE56F19D7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{838775E4-F5E0-431D-9351-D17AE56F19D7}" name="Line" displayName="Line" ref="R1:R17" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
+  <autoFilter ref="R1:R17" xr:uid="{838775E4-F5E0-431D-9351-D17AE56F19D7}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{8390CAA7-046C-4F7E-8958-FFCCA51C7490}" name="Line" dataDxfId="14" dataCellStyle="Normální 2"/>
   </tableColumns>
@@ -3757,8 +4264,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{6464D72C-C69A-4112-8424-97766E88D7C7}" name="S_SMS" displayName="S_SMS" ref="I1:I6" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42" headerRowCellStyle="Normální 2">
-  <autoFilter ref="I1:I6" xr:uid="{6464D72C-C69A-4112-8424-97766E88D7C7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{6464D72C-C69A-4112-8424-97766E88D7C7}" name="S_SMS" displayName="S_SMS" ref="I1:I3" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42" headerRowCellStyle="Normální 2">
+  <autoFilter ref="I1:I3" xr:uid="{6464D72C-C69A-4112-8424-97766E88D7C7}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{139A78FA-5925-4655-AE99-194FDAFDFE73}" name="S/SMS" dataDxfId="41"/>
   </tableColumns>
@@ -4096,6 +4603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB1CF6A9-7DDA-404E-90FB-FA3DB2C74227}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AD3506"/>
   <sheetFormatPr defaultColWidth="7.109375" defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
@@ -4120,46 +4628,46 @@
   <sheetData>
     <row r="1" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="57" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>6</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>7</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="O1" s="4" t="s">
         <v>8</v>
@@ -4171,7 +4679,7 @@
         <v>9</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="S1" s="3" t="s">
         <v>10</v>
@@ -4179,19 +4687,19 @@
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="F2" s="8">
         <v>1</v>
@@ -4202,11 +4710,11 @@
       <c r="H2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="69" t="s">
-        <v>13</v>
+      <c r="I2" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K2" s="5" t="s">
         <v>15</v>
@@ -4226,7 +4734,7 @@
       <c r="P2" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="Q2" s="70" t="s">
+      <c r="Q2" s="59" t="s">
         <v>21</v>
       </c>
       <c r="R2" s="7" t="s">
@@ -4238,19 +4746,19 @@
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="F3" s="8">
         <v>1</v>
@@ -4262,7 +4770,7 @@
         <v>25</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>27</v>
@@ -4285,7 +4793,7 @@
       <c r="P3" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="Q3" s="70" t="s">
+      <c r="Q3" s="59" t="s">
         <v>33</v>
       </c>
       <c r="R3" s="7" t="s">
@@ -4297,19 +4805,19 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="F4" s="8">
         <v>0.99</v>
@@ -4320,285 +4828,276 @@
       <c r="H4" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="I4" s="69" t="s">
-        <v>38</v>
-      </c>
       <c r="J4" s="5" t="s">
         <v>14</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="L4" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M4" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="N4" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="N4" s="5" t="s">
+      <c r="O4" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="P4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="P4" s="7" t="s">
+      <c r="Q4" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="Q4" s="7" t="s">
+      <c r="R4" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="R4" s="7" t="s">
+      <c r="S4" s="5" t="s">
         <v>46</v>
-      </c>
-      <c r="S4" s="5" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="F5" s="8">
         <v>1</v>
       </c>
       <c r="G5" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="K5" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="I5" s="69" t="s">
+      <c r="L5" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="K5" s="5" t="s">
+      <c r="M5" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="N5" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="L5" s="7" t="s">
+      <c r="O5" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="M5" s="5" t="s">
-        <v>390</v>
-      </c>
-      <c r="N5" s="5" t="s">
+      <c r="P5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="Q5" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="R5" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="Q5" s="7" t="s">
+      <c r="S5" s="5" t="s">
         <v>56</v>
-      </c>
-      <c r="R5" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="S5" s="5" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="F6" s="8">
         <v>0.5</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="I6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="M6" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="K6" s="5" t="s">
-        <v>432</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>444</v>
-      </c>
-      <c r="M6" s="5" t="s">
+      <c r="N6" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="O6" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="N6" s="5" t="s">
+      <c r="P6" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="Q6" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="P6" s="7" t="s">
+      <c r="R6" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="Q6" s="7" t="s">
+      <c r="S6" s="5" t="s">
         <v>67</v>
-      </c>
-      <c r="R6" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="S6" s="5" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="F7" s="8">
         <v>1</v>
       </c>
       <c r="G7" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="M7" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="H7" s="5" t="s">
-        <v>276</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="L7" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="M7" s="5" t="s">
+      <c r="N7" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="O7" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="P7" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="R7" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="P7" s="7" t="s">
+      <c r="S7" s="5" t="s">
         <v>75</v>
-      </c>
-      <c r="R7" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="S7" s="5" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="F8" s="8">
         <v>1</v>
       </c>
       <c r="G8" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>443</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="O8" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="K8" s="5" t="s">
-        <v>434</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>445</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>391</v>
-      </c>
-      <c r="N8" s="5" t="s">
+      <c r="P8" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="O8" s="7" t="s">
+      <c r="R8" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="P8" s="7" t="s">
+      <c r="S8" s="5" t="s">
         <v>81</v>
-      </c>
-      <c r="R8" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="S8" s="5" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="F9" s="8">
         <v>0.45</v>
       </c>
       <c r="G9" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="M9" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="K9" s="5" t="s">
-        <v>435</v>
-      </c>
-      <c r="L9" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="M9" s="5" t="s">
+      <c r="N9" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="O9" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="N9" s="5" t="s">
+      <c r="P9" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="R9" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="P9" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="R9" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="S9" s="5" t="s">
         <v>15</v>
@@ -4606,1135 +5105,1141 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="F10" s="8">
         <v>0.94</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="O10" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="P10" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="R10" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="P10" s="7" t="s">
+      <c r="S10" s="5" t="s">
         <v>95</v>
-      </c>
-      <c r="R10" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="S10" s="5" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="F11" s="8">
         <v>0.43</v>
       </c>
       <c r="G11" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="N11" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="O11" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="K11" s="5" t="s">
-        <v>437</v>
-      </c>
-      <c r="L11" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="M11" s="5" t="s">
-        <v>389</v>
-      </c>
-      <c r="N11" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="O11" s="7" t="s">
+      <c r="P11" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="R11" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="P11" s="7" t="s">
+      <c r="S11" s="5" t="s">
         <v>101</v>
-      </c>
-      <c r="R11" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="S11" s="5" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="F12" s="8">
         <v>0.5</v>
       </c>
       <c r="G12" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="M12" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="K12" s="5" t="s">
-        <v>438</v>
-      </c>
-      <c r="L12" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="M12" s="5" t="s">
+      <c r="N12" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="O12" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="P12" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="N12" s="7" t="s">
-        <v>276</v>
-      </c>
-      <c r="O12" s="7" t="s">
+      <c r="R12" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="P12" s="7" t="s">
+      <c r="S12" s="5" t="s">
         <v>108</v>
-      </c>
-      <c r="R12" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="S12" s="5" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F13" s="8">
         <v>0.5</v>
       </c>
       <c r="G13" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M13" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="K13" s="5" t="s">
-        <v>439</v>
-      </c>
-      <c r="L13" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="M13" s="5" t="s">
+      <c r="O13" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="P13" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="O13" s="7" t="s">
+      <c r="R13" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="P13" s="7" t="s">
+      <c r="S13" s="5" t="s">
         <v>115</v>
-      </c>
-      <c r="R13" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="S13" s="5" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="F14" s="8">
         <v>0.76</v>
       </c>
       <c r="G14" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="M14" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="O14" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="K14" s="5" t="s">
-        <v>440</v>
-      </c>
-      <c r="L14" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="M14" s="5" t="s">
-        <v>446</v>
-      </c>
-      <c r="O14" s="7" t="s">
+      <c r="P14" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="R14" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="P14" s="7" t="s">
+      <c r="S14" s="5" t="s">
         <v>121</v>
-      </c>
-      <c r="R14" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="S14" s="5" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="F15" s="8">
         <v>0.96</v>
       </c>
       <c r="G15" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="M15" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="P15" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="K15" s="5" t="s">
-        <v>441</v>
-      </c>
-      <c r="L15" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="M15" s="5" t="s">
-        <v>447</v>
-      </c>
-      <c r="P15" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="R15" s="7"/>
+      <c r="R15" s="7" t="s">
+        <v>451</v>
+      </c>
       <c r="S15" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="F16" s="8">
         <v>0.19</v>
       </c>
       <c r="G16" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="M16" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="P16" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="K16" s="5" t="s">
-        <v>442</v>
-      </c>
-      <c r="L16" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="M16" s="5" t="s">
-        <v>448</v>
-      </c>
-      <c r="P16" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="R16" s="7"/>
+      <c r="R16" s="7" t="s">
+        <v>450</v>
+      </c>
       <c r="S16" s="5" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="F17" s="8">
         <v>0.2</v>
       </c>
       <c r="G17" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="M17" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="P17" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="K17" s="5" t="s">
-        <v>443</v>
-      </c>
-      <c r="L17" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="M17" s="5" t="s">
+      <c r="R17" s="7" t="s">
         <v>449</v>
       </c>
-      <c r="P17" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="R17" s="7"/>
       <c r="S17" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="F18" s="8">
         <v>0.6</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="M18" s="58"/>
       <c r="P18" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="R18" s="7"/>
       <c r="S18" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="19" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="F19" s="8">
         <v>1</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="M19" s="58"/>
       <c r="P19" s="7" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="R19" s="7"/>
       <c r="S19" s="5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="20" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="F20" s="8">
         <v>0.03</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M20" s="58"/>
       <c r="P20" s="7" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="R20" s="7"/>
       <c r="S20" s="5" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="21" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="F21" s="8">
         <v>0.7</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="M21" s="58"/>
       <c r="P21" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="R21" s="7"/>
     </row>
     <row r="22" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="5" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="L22" s="58"/>
       <c r="M22" s="58"/>
       <c r="P22" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="R22" s="7"/>
     </row>
     <row r="23" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L23" s="58"/>
       <c r="M23" s="58"/>
       <c r="P23" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="R23" s="7"/>
     </row>
     <row r="24" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="5" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="L24" s="58"/>
       <c r="M24" s="58"/>
       <c r="P24" s="7" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="R24" s="7"/>
     </row>
     <row r="25" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="5" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="L25" s="58"/>
       <c r="M25" s="58"/>
       <c r="P25" s="7" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="R25" s="7"/>
     </row>
     <row r="26" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="L26" s="58"/>
       <c r="M26" s="58"/>
       <c r="P26" s="7" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="R26" s="7"/>
     </row>
     <row r="27" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="5" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="L27" s="58"/>
       <c r="P27" s="7" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="R27" s="7"/>
     </row>
     <row r="28" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="5" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="L28" s="58"/>
       <c r="P28" s="7" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="R28" s="7"/>
     </row>
     <row r="29" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="5" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="L29" s="58"/>
       <c r="P29" s="7" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="R29" s="7"/>
     </row>
     <row r="30" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="5" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="L30" s="58"/>
       <c r="P30" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R30" s="7"/>
     </row>
     <row r="31" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="5" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="L31" s="58"/>
       <c r="P31" s="7" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="R31" s="7"/>
     </row>
     <row r="32" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C32" s="5" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="5" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="L32" s="58"/>
       <c r="P32" s="7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="R32" s="7"/>
     </row>
     <row r="33" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C33" s="5" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="5" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="L33" s="58"/>
       <c r="P33" s="7" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="R33" s="7"/>
     </row>
     <row r="34" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C34" s="5" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="L34" s="58"/>
       <c r="P34" s="7" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="R34" s="7"/>
     </row>
     <row r="35" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C35" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="L35" s="58"/>
       <c r="P35" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="R35" s="7"/>
     </row>
     <row r="36" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C36" s="5" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="L36" s="58"/>
       <c r="P36" s="7" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="R36" s="7"/>
     </row>
     <row r="37" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C37" s="5" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="F37" s="6"/>
       <c r="G37" s="5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="L37" s="58"/>
       <c r="P37" s="7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="R37" s="7"/>
     </row>
     <row r="38" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C38" s="5" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="5" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="L38" s="58"/>
       <c r="P38" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="R38" s="7"/>
     </row>
     <row r="39" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C39" s="5" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="F39" s="6"/>
       <c r="G39" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="L39" s="58"/>
       <c r="P39" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="R39" s="7"/>
     </row>
     <row r="40" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C40" s="5" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="L40" s="58"/>
       <c r="P40" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="R40" s="7"/>
     </row>
     <row r="41" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C41" s="5" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="5" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="L41" s="58"/>
       <c r="P41" s="7" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="R41" s="7"/>
     </row>
     <row r="42" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C42" s="5" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F42" s="6"/>
       <c r="G42" s="5" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="L42" s="7"/>
       <c r="P42" s="7" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="R42" s="7"/>
     </row>
     <row r="43" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C43" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="F43" s="6"/>
       <c r="G43" s="5" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="L43" s="7"/>
       <c r="P43" s="7" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="R43" s="7"/>
     </row>
     <row r="44" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C44" s="5" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="F44" s="6"/>
       <c r="G44" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="L44" s="7"/>
       <c r="P44" s="7" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="R44" s="7"/>
     </row>
     <row r="45" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C45" s="5" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="F45" s="6"/>
       <c r="G45" s="5" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="L45" s="7"/>
       <c r="P45" s="7" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="R45" s="7"/>
     </row>
     <row r="46" spans="3:18" x14ac:dyDescent="0.2">
       <c r="F46" s="6"/>
       <c r="G46" s="5" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="L46" s="7"/>
       <c r="P46" s="7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="R46" s="7"/>
     </row>
     <row r="47" spans="3:18" x14ac:dyDescent="0.2">
       <c r="F47" s="6"/>
       <c r="G47" s="5" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="L47" s="7"/>
       <c r="P47" s="7" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="R47" s="7"/>
     </row>
     <row r="48" spans="3:18" x14ac:dyDescent="0.2">
       <c r="F48" s="6"/>
       <c r="G48" s="5" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="L48" s="7"/>
       <c r="P48" s="7" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="R48" s="7"/>
     </row>
     <row r="49" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F49" s="6"/>
       <c r="G49" s="5" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L49" s="7"/>
       <c r="P49" s="7" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="R49" s="7"/>
     </row>
     <row r="50" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F50" s="6"/>
       <c r="G50" s="5" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L50" s="7"/>
       <c r="P50" s="7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="R50" s="7"/>
     </row>
     <row r="51" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F51" s="6"/>
       <c r="G51" s="5" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L51" s="7"/>
       <c r="P51" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="R51" s="7"/>
     </row>
     <row r="52" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F52" s="6"/>
       <c r="G52" s="5" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="L52" s="7"/>
       <c r="P52" s="7" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="R52" s="7"/>
     </row>
     <row r="53" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F53" s="6"/>
       <c r="G53" s="5" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="L53" s="7"/>
       <c r="P53" s="7" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="R53" s="7"/>
     </row>
     <row r="54" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F54" s="6"/>
       <c r="G54" s="5" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="L54" s="7"/>
       <c r="P54" s="7" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="R54" s="7"/>
     </row>
     <row r="55" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F55" s="6"/>
       <c r="G55" s="5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="L55" s="7"/>
       <c r="P55" s="7" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="R55" s="7"/>
     </row>
     <row r="56" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F56" s="6"/>
       <c r="G56" s="5" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L56" s="7"/>
       <c r="P56" s="7" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="R56" s="7"/>
     </row>
     <row r="57" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F57" s="6"/>
       <c r="G57" s="5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="L57" s="7"/>
       <c r="P57" s="7" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="R57" s="7"/>
     </row>
     <row r="58" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F58" s="6"/>
       <c r="G58" s="5" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="L58" s="7"/>
       <c r="P58" s="7" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="R58" s="7"/>
     </row>
     <row r="59" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F59" s="6"/>
       <c r="G59" s="5" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="L59" s="7"/>
       <c r="P59" s="7" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="R59" s="7"/>
     </row>
     <row r="60" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F60" s="6"/>
       <c r="G60" s="5" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="L60" s="7"/>
       <c r="P60" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="R60" s="7"/>
     </row>
     <row r="61" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F61" s="6"/>
       <c r="G61" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="L61" s="7"/>
       <c r="P61" s="7" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="R61" s="7"/>
     </row>
     <row r="62" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F62" s="6"/>
       <c r="G62" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="L62" s="7"/>
       <c r="P62" s="7" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="R62" s="7"/>
     </row>
     <row r="63" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F63" s="6"/>
       <c r="G63" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="L63" s="7"/>
       <c r="P63" s="7" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="R63" s="7"/>
     </row>
     <row r="64" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F64" s="6"/>
       <c r="G64" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="L64" s="7"/>
       <c r="P64" s="7" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="R64" s="7"/>
     </row>
     <row r="65" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F65" s="6"/>
       <c r="G65" s="5" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L65" s="7"/>
       <c r="P65" s="7" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="R65" s="7"/>
     </row>
     <row r="66" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F66" s="6"/>
       <c r="G66" s="5" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="L66" s="7"/>
       <c r="P66" s="7" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="R66" s="7"/>
     </row>
     <row r="67" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F67" s="6"/>
       <c r="G67" s="5" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="L67" s="7"/>
       <c r="P67" s="7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="R67" s="7"/>
     </row>
     <row r="68" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F68" s="6"/>
       <c r="G68" s="5" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="L68" s="7"/>
       <c r="P68" s="7" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="R68" s="7"/>
     </row>
     <row r="69" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F69" s="6"/>
       <c r="G69" s="5" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="L69" s="7"/>
       <c r="P69" s="7" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="R69" s="7"/>
     </row>
     <row r="70" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F70" s="6"/>
       <c r="G70" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="L70" s="7"/>
       <c r="P70" s="7" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="R70" s="7"/>
     </row>
     <row r="71" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F71" s="6"/>
       <c r="G71" s="5" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L71" s="7"/>
       <c r="P71" s="7" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="R71" s="7"/>
     </row>
     <row r="72" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F72" s="6"/>
       <c r="G72" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="L72" s="7"/>
       <c r="P72" s="7" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="R72" s="7"/>
     </row>
     <row r="73" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F73" s="6"/>
       <c r="G73" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="L73" s="7"/>
       <c r="P73" s="7" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="R73" s="7"/>
     </row>
     <row r="74" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F74" s="6"/>
       <c r="G74" s="5" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="L74" s="7"/>
       <c r="P74" s="7" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="R74" s="7"/>
     </row>
     <row r="75" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F75" s="6"/>
       <c r="G75" s="5" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="L75" s="7"/>
       <c r="R75" s="7"/>
@@ -5742,7 +6247,7 @@
     <row r="76" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F76" s="6"/>
       <c r="G76" s="5" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="L76" s="7"/>
       <c r="R76" s="7"/>
@@ -5750,7 +6255,7 @@
     <row r="77" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F77" s="6"/>
       <c r="G77" s="5" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="L77" s="7"/>
       <c r="R77" s="7"/>
@@ -5758,7 +6263,7 @@
     <row r="78" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F78" s="6"/>
       <c r="G78" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="L78" s="7"/>
       <c r="R78" s="7"/>
@@ -5766,7 +6271,7 @@
     <row r="79" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F79" s="6"/>
       <c r="G79" s="5" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="L79" s="7"/>
       <c r="R79" s="7"/>
@@ -5774,7 +6279,7 @@
     <row r="80" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F80" s="6"/>
       <c r="G80" s="5" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="L80" s="7"/>
       <c r="R80" s="7"/>
@@ -5782,7 +6287,7 @@
     <row r="81" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F81" s="6"/>
       <c r="G81" s="5" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="L81" s="7"/>
       <c r="R81" s="7"/>
@@ -5790,7 +6295,7 @@
     <row r="82" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F82" s="6"/>
       <c r="G82" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="L82" s="7"/>
       <c r="R82" s="7"/>
@@ -5798,7 +6303,7 @@
     <row r="83" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F83" s="6"/>
       <c r="G83" s="5" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="L83" s="7"/>
       <c r="R83" s="7"/>
@@ -5806,7 +6311,7 @@
     <row r="84" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F84" s="6"/>
       <c r="G84" s="5" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="L84" s="7"/>
       <c r="R84" s="7"/>
@@ -5814,7 +6319,7 @@
     <row r="85" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F85" s="6"/>
       <c r="G85" s="5" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="L85" s="7"/>
       <c r="R85" s="7"/>
@@ -5822,7 +6327,7 @@
     <row r="86" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F86" s="6"/>
       <c r="G86" s="5" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="L86" s="7"/>
       <c r="R86" s="7"/>
@@ -5830,7 +6335,7 @@
     <row r="87" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F87" s="6"/>
       <c r="G87" s="5" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="L87" s="7"/>
       <c r="R87" s="7"/>
@@ -5904,6 +6409,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE2A24B-6F86-49F0-A1AD-597518264221}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AA29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -5921,7 +6427,7 @@
     <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" s="9"/>
       <c r="B1" s="10" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="C1" s="9"/>
       <c r="D1" s="9"/>
@@ -5956,7 +6462,7 @@
         <v>1000</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E2" s="9"/>
       <c r="F2" s="9"/>
@@ -5985,14 +6491,14 @@
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" s="10"/>
       <c r="B3" s="10"/>
-      <c r="C3" s="63" t="s">
-        <v>268</v>
-      </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="63" t="s">
-        <v>268</v>
-      </c>
-      <c r="F3" s="64"/>
+      <c r="C3" s="78" t="s">
+        <v>266</v>
+      </c>
+      <c r="D3" s="79"/>
+      <c r="E3" s="78" t="s">
+        <v>266</v>
+      </c>
+      <c r="F3" s="79"/>
       <c r="G3" s="14" t="s">
         <v>13</v>
       </c>
@@ -6005,14 +6511,14 @@
       <c r="J3" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="K3" s="65" t="s">
-        <v>268</v>
-      </c>
-      <c r="L3" s="66"/>
-      <c r="M3" s="63" t="s">
-        <v>268</v>
-      </c>
-      <c r="N3" s="64"/>
+      <c r="K3" s="80" t="s">
+        <v>266</v>
+      </c>
+      <c r="L3" s="81"/>
+      <c r="M3" s="78" t="s">
+        <v>266</v>
+      </c>
+      <c r="N3" s="79"/>
       <c r="O3" s="9"/>
       <c r="P3" s="9"/>
       <c r="Q3" s="13"/>
@@ -6029,37 +6535,37 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="B4" s="16"/>
+      <c r="C4" s="82" t="s">
+        <v>394</v>
+      </c>
+      <c r="D4" s="83"/>
+      <c r="E4" s="82" t="s">
         <v>395</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="67" t="s">
+      <c r="F4" s="83"/>
+      <c r="G4" s="17" t="s">
         <v>396</v>
       </c>
-      <c r="D4" s="68"/>
-      <c r="E4" s="67" t="s">
+      <c r="H4" s="15" t="s">
         <v>397</v>
       </c>
-      <c r="F4" s="68"/>
-      <c r="G4" s="17" t="s">
+      <c r="I4" s="17" t="s">
         <v>398</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="J4" s="15" t="s">
         <v>399</v>
       </c>
-      <c r="I4" s="17" t="s">
+      <c r="K4" s="82" t="s">
         <v>400</v>
       </c>
-      <c r="J4" s="15" t="s">
+      <c r="L4" s="83"/>
+      <c r="M4" s="82" t="s">
         <v>401</v>
       </c>
-      <c r="K4" s="67" t="s">
-        <v>402</v>
-      </c>
-      <c r="L4" s="68"/>
-      <c r="M4" s="67" t="s">
-        <v>403</v>
-      </c>
-      <c r="N4" s="68"/>
+      <c r="N4" s="83"/>
       <c r="O4" s="9"/>
       <c r="P4" s="9"/>
       <c r="Q4" s="9"/>
@@ -6076,25 +6582,25 @@
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B5" s="18"/>
-      <c r="C5" s="59">
+      <c r="C5" s="84">
         <v>34.700000000000003</v>
       </c>
-      <c r="D5" s="60"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="60"/>
+      <c r="D5" s="85"/>
+      <c r="E5" s="84"/>
+      <c r="F5" s="85"/>
       <c r="G5" s="19">
         <v>5.3</v>
       </c>
       <c r="H5" s="20"/>
       <c r="I5" s="19"/>
       <c r="J5" s="19"/>
-      <c r="K5" s="59"/>
-      <c r="L5" s="60"/>
-      <c r="M5" s="59"/>
-      <c r="N5" s="60"/>
+      <c r="K5" s="84"/>
+      <c r="L5" s="85"/>
+      <c r="M5" s="84"/>
+      <c r="N5" s="85"/>
       <c r="O5" s="21">
         <f>SUM(C5:N5)</f>
         <v>40</v>
@@ -6114,19 +6620,19 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" s="25" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="B6" s="25"/>
-      <c r="C6" s="61">
+      <c r="C6" s="86">
         <f>C5/$O$5</f>
         <v>0.86750000000000005</v>
       </c>
-      <c r="D6" s="62"/>
-      <c r="E6" s="61">
+      <c r="D6" s="87"/>
+      <c r="E6" s="86">
         <f>E5/$O$5</f>
         <v>0</v>
       </c>
-      <c r="F6" s="62"/>
+      <c r="F6" s="87"/>
       <c r="G6" s="26">
         <f>G5/$O$5</f>
         <v>0.13250000000000001</v>
@@ -6143,16 +6649,16 @@
         <f>J5/$O$5</f>
         <v>0</v>
       </c>
-      <c r="K6" s="61">
+      <c r="K6" s="86">
         <f>K5/$O$5</f>
         <v>0</v>
       </c>
-      <c r="L6" s="62"/>
-      <c r="M6" s="61">
+      <c r="L6" s="87"/>
+      <c r="M6" s="86">
         <f>M5/$O$5</f>
         <v>0</v>
       </c>
-      <c r="N6" s="62"/>
+      <c r="N6" s="87"/>
       <c r="O6" s="27">
         <f>SUM(C6:N6)</f>
         <v>1</v>
@@ -6172,44 +6678,44 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" s="29" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B7" s="29"/>
       <c r="C7" s="30" t="s">
+        <v>405</v>
+      </c>
+      <c r="D7" s="30" t="s">
+        <v>406</v>
+      </c>
+      <c r="E7" s="30" t="s">
+        <v>405</v>
+      </c>
+      <c r="F7" s="30" t="s">
+        <v>406</v>
+      </c>
+      <c r="G7" s="30" t="s">
         <v>407</v>
       </c>
-      <c r="D7" s="30" t="s">
-        <v>408</v>
-      </c>
-      <c r="E7" s="30" t="s">
+      <c r="H7" s="30" t="s">
         <v>407</v>
       </c>
-      <c r="F7" s="30" t="s">
-        <v>408</v>
-      </c>
-      <c r="G7" s="30" t="s">
-        <v>409</v>
-      </c>
-      <c r="H7" s="30" t="s">
-        <v>409</v>
-      </c>
       <c r="I7" s="30" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="J7" s="30" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="K7" s="30" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="L7" s="30" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="M7" s="30" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="N7" s="30" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="O7" s="9"/>
       <c r="P7" s="9"/>
@@ -6227,7 +6733,7 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" s="29" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B8" s="29"/>
       <c r="C8" s="32">
@@ -6325,7 +6831,7 @@
         <v>0</v>
       </c>
       <c r="B10" s="32" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C10" s="32">
         <v>1</v>
@@ -6407,7 +6913,7 @@
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="B12" s="32"/>
       <c r="C12" s="37"/>
@@ -6482,7 +6988,7 @@
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" s="29" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B14" s="32"/>
       <c r="C14" s="37"/>
@@ -6555,10 +7061,10 @@
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" s="29" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B16" s="32" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C16" s="37">
         <v>7.0000000000000001E-3</v>
@@ -6590,7 +7096,7 @@
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A17" s="29" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B17" s="32"/>
       <c r="C17" s="37"/>
@@ -6621,7 +7127,7 @@
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A18" s="29" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="B18" s="32"/>
       <c r="C18" s="37"/>
@@ -6652,7 +7158,7 @@
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A19" s="29" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B19" s="32"/>
       <c r="C19" s="37"/>
@@ -6683,7 +7189,7 @@
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A20" s="29" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="B20" s="32"/>
       <c r="C20" s="37"/>
@@ -6745,13 +7251,13 @@
       <c r="A22" s="41"/>
       <c r="B22" s="42"/>
       <c r="C22" s="43" t="s">
+        <v>416</v>
+      </c>
+      <c r="D22" s="43" t="s">
+        <v>417</v>
+      </c>
+      <c r="E22" s="44" t="s">
         <v>418</v>
-      </c>
-      <c r="D22" s="43" t="s">
-        <v>419</v>
-      </c>
-      <c r="E22" s="44" t="s">
-        <v>420</v>
       </c>
       <c r="F22" s="45"/>
       <c r="G22" s="45"/>
@@ -6778,10 +7284,10 @@
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A23" s="29" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="B23" s="32" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C23" s="35">
         <f>_xlfn.XLOOKUP(B23,Surfactant[Surfactant],Surfactant[Surf_conc.])</f>
@@ -6819,7 +7325,7 @@
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A24" s="29" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B24" s="32"/>
       <c r="C24" s="35" t="e">
@@ -6856,7 +7362,7 @@
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A25" s="29" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="B25" s="32"/>
       <c r="C25" s="35" t="e">
@@ -6925,76 +7431,76 @@
         <v>0</v>
       </c>
       <c r="B27" s="48" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="C27" s="48" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="D27" s="48" t="s">
         <v>1</v>
       </c>
       <c r="E27" s="48" t="s">
+        <v>411</v>
+      </c>
+      <c r="F27" s="48" t="s">
+        <v>412</v>
+      </c>
+      <c r="G27" s="48" t="s">
         <v>413</v>
       </c>
-      <c r="F27" s="48" t="s">
+      <c r="H27" s="48" t="s">
         <v>414</v>
       </c>
-      <c r="G27" s="48" t="s">
+      <c r="I27" s="48" t="s">
         <v>415</v>
       </c>
-      <c r="H27" s="48" t="s">
-        <v>416</v>
-      </c>
-      <c r="I27" s="48" t="s">
-        <v>417</v>
-      </c>
       <c r="J27" s="48" t="s">
+        <v>419</v>
+      </c>
+      <c r="K27" s="48" t="s">
+        <v>420</v>
+      </c>
+      <c r="L27" s="48" t="s">
         <v>421</v>
-      </c>
-      <c r="K27" s="48" t="s">
-        <v>422</v>
-      </c>
-      <c r="L27" s="48" t="s">
-        <v>423</v>
       </c>
       <c r="M27" s="48" t="s">
         <v>0</v>
       </c>
       <c r="N27" s="48" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="O27" s="48" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="P27" s="48" t="s">
         <v>1</v>
       </c>
       <c r="Q27" s="48" t="s">
+        <v>411</v>
+      </c>
+      <c r="R27" s="48" t="s">
+        <v>412</v>
+      </c>
+      <c r="S27" s="48" t="s">
         <v>413</v>
       </c>
-      <c r="R27" s="48" t="s">
+      <c r="T27" s="48" t="s">
         <v>414</v>
       </c>
-      <c r="S27" s="48" t="s">
+      <c r="U27" s="48" t="s">
         <v>415</v>
       </c>
-      <c r="T27" s="48" t="s">
-        <v>416</v>
-      </c>
-      <c r="U27" s="48" t="s">
+      <c r="V27" s="48" t="s">
+        <v>419</v>
+      </c>
+      <c r="W27" s="48" t="s">
+        <v>420</v>
+      </c>
+      <c r="X27" s="48" t="s">
+        <v>421</v>
+      </c>
+      <c r="Y27" s="48" t="s">
         <v>417</v>
-      </c>
-      <c r="V27" s="48" t="s">
-        <v>421</v>
-      </c>
-      <c r="W27" s="48" t="s">
-        <v>422</v>
-      </c>
-      <c r="X27" s="48" t="s">
-        <v>423</v>
-      </c>
-      <c r="Y27" s="48" t="s">
-        <v>419</v>
       </c>
       <c r="Z27" s="22"/>
       <c r="AA27" s="22"/>
@@ -7152,6 +7658,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="M5:N5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="M6:N6"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="K3:L3"/>
@@ -7160,14 +7674,6 @@
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="K4:L4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="M5:N5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="M6:N6"/>
   </mergeCells>
   <conditionalFormatting sqref="A29">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="notEqual">
@@ -7206,7 +7712,7 @@
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
             <control shapeId="2049" r:id="rId3" name="Button 1">
-              <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="[1]!výmaz">
+              <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0">
                 <anchor moveWithCells="1" sizeWithCells="1">
                   <from>
                     <xdr:col>0</xdr:col>
@@ -7241,4 +7747,869 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76C66FB5-2B4A-4875-9FDB-3206A3D6438C}">
+  <dimension ref="B2:Y16"/>
+  <sheetFormatPr defaultColWidth="6.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="1.109375" style="73" customWidth="1"/>
+    <col min="2" max="2" width="5" style="73" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" style="73" customWidth="1"/>
+    <col min="4" max="4" width="7" style="73" customWidth="1"/>
+    <col min="5" max="5" width="13.109375" style="73" customWidth="1"/>
+    <col min="6" max="12" width="12.77734375" style="73" customWidth="1"/>
+    <col min="13" max="13" width="19.44140625" style="73" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.109375" style="73" bestFit="1" customWidth="1"/>
+    <col min="15" max="19" width="8.5546875" style="73" customWidth="1"/>
+    <col min="20" max="20" width="9.6640625" style="73" customWidth="1"/>
+    <col min="21" max="21" width="11.21875" style="73" customWidth="1"/>
+    <col min="22" max="22" width="14.5546875" style="73" customWidth="1"/>
+    <col min="23" max="23" width="12" style="73" customWidth="1"/>
+    <col min="24" max="24" width="9.21875" style="73" customWidth="1"/>
+    <col min="25" max="25" width="10.6640625" style="73" customWidth="1"/>
+    <col min="26" max="16384" width="6.5546875" style="73"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:25" s="62" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="B2" s="60" t="s">
+        <v>452</v>
+      </c>
+      <c r="C2" s="60" t="s">
+        <v>453</v>
+      </c>
+      <c r="D2" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="E2" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="F2" s="61"/>
+      <c r="G2" s="74" t="s">
+        <v>456</v>
+      </c>
+      <c r="H2" s="75"/>
+      <c r="I2" s="75"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="75"/>
+      <c r="L2" s="76"/>
+      <c r="M2" s="60" t="s">
+        <v>457</v>
+      </c>
+      <c r="N2" s="60" t="s">
+        <v>458</v>
+      </c>
+      <c r="O2" s="74" t="s">
+        <v>459</v>
+      </c>
+      <c r="P2" s="76"/>
+      <c r="Q2" s="74" t="s">
+        <v>460</v>
+      </c>
+      <c r="R2" s="76"/>
+      <c r="S2" s="74" t="s">
+        <v>461</v>
+      </c>
+      <c r="T2" s="76"/>
+      <c r="U2" s="60" t="s">
+        <v>462</v>
+      </c>
+      <c r="V2" s="60" t="s">
+        <v>463</v>
+      </c>
+      <c r="W2" s="60" t="s">
+        <v>464</v>
+      </c>
+      <c r="X2" s="60" t="s">
+        <v>465</v>
+      </c>
+      <c r="Y2" s="60" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="3" spans="2:25" s="62" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60" t="s">
+        <v>467</v>
+      </c>
+      <c r="G3" s="60" t="s">
+        <v>468</v>
+      </c>
+      <c r="H3" s="60" t="s">
+        <v>469</v>
+      </c>
+      <c r="I3" s="60" t="s">
+        <v>470</v>
+      </c>
+      <c r="J3" s="60" t="s">
+        <v>471</v>
+      </c>
+      <c r="K3" s="60" t="s">
+        <v>472</v>
+      </c>
+      <c r="L3" s="60" t="s">
+        <v>473</v>
+      </c>
+      <c r="M3" s="60" t="s">
+        <v>474</v>
+      </c>
+      <c r="N3" s="60" t="s">
+        <v>474</v>
+      </c>
+      <c r="O3" s="60" t="s">
+        <v>38</v>
+      </c>
+      <c r="P3" s="60" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q3" s="60" t="s">
+        <v>38</v>
+      </c>
+      <c r="R3" s="60" t="s">
+        <v>14</v>
+      </c>
+      <c r="S3" s="60" t="s">
+        <v>38</v>
+      </c>
+      <c r="T3" s="60" t="s">
+        <v>14</v>
+      </c>
+      <c r="U3" s="60" t="s">
+        <v>474</v>
+      </c>
+      <c r="V3" s="60" t="s">
+        <v>474</v>
+      </c>
+      <c r="W3" s="60" t="s">
+        <v>474</v>
+      </c>
+      <c r="X3" s="60" t="s">
+        <v>474</v>
+      </c>
+      <c r="Y3" s="60" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="4" spans="2:25" s="62" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="B4" s="63" t="s">
+        <v>475</v>
+      </c>
+      <c r="C4" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="63">
+        <v>3.3</v>
+      </c>
+      <c r="E4" s="63">
+        <v>3.55</v>
+      </c>
+      <c r="F4" s="63" t="s">
+        <v>476</v>
+      </c>
+      <c r="G4" s="64"/>
+      <c r="H4" s="64"/>
+      <c r="I4" s="64"/>
+      <c r="J4" s="64"/>
+      <c r="K4" s="64"/>
+      <c r="L4" s="64"/>
+      <c r="M4" s="63" t="s">
+        <v>477</v>
+      </c>
+      <c r="N4" s="63" t="s">
+        <v>478</v>
+      </c>
+      <c r="O4" s="63">
+        <v>71</v>
+      </c>
+      <c r="P4" s="64"/>
+      <c r="Q4" s="63">
+        <v>113</v>
+      </c>
+      <c r="R4" s="64"/>
+      <c r="S4" s="63">
+        <v>120</v>
+      </c>
+      <c r="T4" s="64"/>
+      <c r="U4" s="64"/>
+      <c r="V4" s="64"/>
+      <c r="W4" s="64"/>
+      <c r="X4" s="63">
+        <v>24</v>
+      </c>
+      <c r="Y4" s="63" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="5" spans="2:25" s="62" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="B5" s="63" t="s">
+        <v>480</v>
+      </c>
+      <c r="C5" s="63" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" s="63">
+        <v>3.3</v>
+      </c>
+      <c r="E5" s="63">
+        <v>3.6</v>
+      </c>
+      <c r="F5" s="63" t="s">
+        <v>481</v>
+      </c>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="63" t="s">
+        <v>482</v>
+      </c>
+      <c r="J5" s="64"/>
+      <c r="K5" s="64"/>
+      <c r="L5" s="64"/>
+      <c r="M5" s="63" t="s">
+        <v>483</v>
+      </c>
+      <c r="N5" s="63" t="s">
+        <v>484</v>
+      </c>
+      <c r="O5" s="63">
+        <v>97</v>
+      </c>
+      <c r="P5" s="64"/>
+      <c r="Q5" s="63">
+        <v>106</v>
+      </c>
+      <c r="R5" s="64"/>
+      <c r="S5" s="63">
+        <v>126</v>
+      </c>
+      <c r="T5" s="64"/>
+      <c r="U5" s="63">
+        <v>17</v>
+      </c>
+      <c r="V5" s="63">
+        <v>35</v>
+      </c>
+      <c r="W5" s="63">
+        <v>60</v>
+      </c>
+      <c r="X5" s="63">
+        <v>40</v>
+      </c>
+      <c r="Y5" s="65" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="6" spans="2:25" s="62" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="B6" s="63" t="s">
+        <v>486</v>
+      </c>
+      <c r="C6" s="63" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="63">
+        <v>3.5</v>
+      </c>
+      <c r="E6" s="63">
+        <v>3.8</v>
+      </c>
+      <c r="F6" s="63" t="s">
+        <v>487</v>
+      </c>
+      <c r="G6" s="63" t="s">
+        <v>488</v>
+      </c>
+      <c r="H6" s="64"/>
+      <c r="I6" s="63" t="s">
+        <v>489</v>
+      </c>
+      <c r="J6" s="64"/>
+      <c r="K6" s="64"/>
+      <c r="L6" s="64"/>
+      <c r="M6" s="63" t="s">
+        <v>490</v>
+      </c>
+      <c r="N6" s="63" t="s">
+        <v>491</v>
+      </c>
+      <c r="O6" s="63">
+        <v>135</v>
+      </c>
+      <c r="P6" s="64"/>
+      <c r="Q6" s="63">
+        <v>155</v>
+      </c>
+      <c r="R6" s="64"/>
+      <c r="S6" s="63">
+        <v>165</v>
+      </c>
+      <c r="T6" s="64"/>
+      <c r="U6" s="63">
+        <v>18</v>
+      </c>
+      <c r="V6" s="63">
+        <v>40</v>
+      </c>
+      <c r="W6" s="63">
+        <v>54.4</v>
+      </c>
+      <c r="X6" s="63">
+        <v>38</v>
+      </c>
+      <c r="Y6" s="63" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="7" spans="2:25" s="62" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="B7" s="60" t="s">
+        <v>493</v>
+      </c>
+      <c r="C7" s="60" t="s">
+        <v>494</v>
+      </c>
+      <c r="D7" s="66">
+        <v>3.5</v>
+      </c>
+      <c r="E7" s="66">
+        <v>3.8</v>
+      </c>
+      <c r="F7" s="66" t="s">
+        <v>495</v>
+      </c>
+      <c r="G7" s="67"/>
+      <c r="H7" s="67"/>
+      <c r="I7" s="66" t="s">
+        <v>496</v>
+      </c>
+      <c r="J7" s="67"/>
+      <c r="K7" s="66" t="s">
+        <v>497</v>
+      </c>
+      <c r="L7" s="66" t="s">
+        <v>498</v>
+      </c>
+      <c r="M7" s="66" t="s">
+        <v>499</v>
+      </c>
+      <c r="N7" s="66" t="s">
+        <v>500</v>
+      </c>
+      <c r="O7" s="66">
+        <v>135</v>
+      </c>
+      <c r="P7" s="66">
+        <v>139</v>
+      </c>
+      <c r="Q7" s="66">
+        <v>155</v>
+      </c>
+      <c r="R7" s="66">
+        <v>155</v>
+      </c>
+      <c r="S7" s="66">
+        <v>162</v>
+      </c>
+      <c r="T7" s="66">
+        <v>160</v>
+      </c>
+      <c r="U7" s="66">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="V7" s="66">
+        <v>40</v>
+      </c>
+      <c r="W7" s="66">
+        <v>54.7</v>
+      </c>
+      <c r="X7" s="66">
+        <v>35</v>
+      </c>
+      <c r="Y7" s="66">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="2:25" s="62" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="B8" s="60" t="s">
+        <v>501</v>
+      </c>
+      <c r="C8" s="60" t="s">
+        <v>502</v>
+      </c>
+      <c r="D8" s="66">
+        <v>3.5</v>
+      </c>
+      <c r="E8" s="66">
+        <v>3.8</v>
+      </c>
+      <c r="F8" s="66" t="s">
+        <v>503</v>
+      </c>
+      <c r="G8" s="66" t="s">
+        <v>504</v>
+      </c>
+      <c r="H8" s="67"/>
+      <c r="I8" s="67"/>
+      <c r="J8" s="67"/>
+      <c r="K8" s="66" t="s">
+        <v>505</v>
+      </c>
+      <c r="L8" s="66" t="s">
+        <v>506</v>
+      </c>
+      <c r="M8" s="66" t="s">
+        <v>507</v>
+      </c>
+      <c r="N8" s="66" t="s">
+        <v>508</v>
+      </c>
+      <c r="O8" s="66">
+        <v>140</v>
+      </c>
+      <c r="P8" s="66">
+        <v>140</v>
+      </c>
+      <c r="Q8" s="66">
+        <v>155</v>
+      </c>
+      <c r="R8" s="66">
+        <v>155</v>
+      </c>
+      <c r="S8" s="66">
+        <v>151</v>
+      </c>
+      <c r="T8" s="66">
+        <v>168</v>
+      </c>
+      <c r="U8" s="67"/>
+      <c r="V8" s="67"/>
+      <c r="W8" s="67"/>
+      <c r="X8" s="66">
+        <v>43</v>
+      </c>
+      <c r="Y8" s="66">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="2:25" s="62" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="B9" s="60" t="s">
+        <v>509</v>
+      </c>
+      <c r="C9" s="60" t="s">
+        <v>502</v>
+      </c>
+      <c r="D9" s="66">
+        <v>4.5</v>
+      </c>
+      <c r="E9" s="66">
+        <v>4.8</v>
+      </c>
+      <c r="F9" s="66" t="s">
+        <v>510</v>
+      </c>
+      <c r="G9" s="66" t="s">
+        <v>511</v>
+      </c>
+      <c r="H9" s="66" t="s">
+        <v>512</v>
+      </c>
+      <c r="I9" s="67"/>
+      <c r="J9" s="67"/>
+      <c r="K9" s="67"/>
+      <c r="L9" s="67"/>
+      <c r="M9" s="66" t="s">
+        <v>513</v>
+      </c>
+      <c r="N9" s="66" t="s">
+        <v>514</v>
+      </c>
+      <c r="O9" s="66">
+        <v>160</v>
+      </c>
+      <c r="P9" s="67"/>
+      <c r="Q9" s="66">
+        <v>220</v>
+      </c>
+      <c r="R9" s="67"/>
+      <c r="S9" s="66">
+        <v>240</v>
+      </c>
+      <c r="T9" s="67"/>
+      <c r="U9" s="67"/>
+      <c r="V9" s="67"/>
+      <c r="W9" s="67"/>
+      <c r="X9" s="66">
+        <v>44</v>
+      </c>
+      <c r="Y9" s="66">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="2:25" s="62" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="B10" s="60" t="s">
+        <v>515</v>
+      </c>
+      <c r="C10" s="60" t="s">
+        <v>516</v>
+      </c>
+      <c r="D10" s="66">
+        <v>3.5</v>
+      </c>
+      <c r="E10" s="66">
+        <v>3.8</v>
+      </c>
+      <c r="F10" s="66" t="s">
+        <v>517</v>
+      </c>
+      <c r="G10" s="66" t="s">
+        <v>518</v>
+      </c>
+      <c r="H10" s="67"/>
+      <c r="I10" s="66" t="s">
+        <v>519</v>
+      </c>
+      <c r="J10" s="66" t="s">
+        <v>520</v>
+      </c>
+      <c r="K10" s="67"/>
+      <c r="L10" s="67"/>
+      <c r="M10" s="66" t="s">
+        <v>521</v>
+      </c>
+      <c r="N10" s="68" t="s">
+        <v>522</v>
+      </c>
+      <c r="O10" s="66">
+        <v>130</v>
+      </c>
+      <c r="P10" s="67"/>
+      <c r="Q10" s="66">
+        <v>200</v>
+      </c>
+      <c r="R10" s="67"/>
+      <c r="S10" s="66">
+        <v>215</v>
+      </c>
+      <c r="T10" s="67"/>
+      <c r="U10" s="66">
+        <v>18</v>
+      </c>
+      <c r="V10" s="66">
+        <v>40</v>
+      </c>
+      <c r="W10" s="66">
+        <v>70</v>
+      </c>
+      <c r="X10" s="66" t="s">
+        <v>523</v>
+      </c>
+      <c r="Y10" s="66">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="2:25" s="62" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="B11" s="60" t="s">
+        <v>524</v>
+      </c>
+      <c r="C11" s="60" t="s">
+        <v>494</v>
+      </c>
+      <c r="D11" s="66">
+        <v>4.7</v>
+      </c>
+      <c r="E11" s="66">
+        <v>5</v>
+      </c>
+      <c r="F11" s="66" t="s">
+        <v>525</v>
+      </c>
+      <c r="G11" s="67"/>
+      <c r="H11" s="67"/>
+      <c r="I11" s="66" t="s">
+        <v>526</v>
+      </c>
+      <c r="J11" s="67"/>
+      <c r="K11" s="66" t="s">
+        <v>527</v>
+      </c>
+      <c r="L11" s="66" t="s">
+        <v>528</v>
+      </c>
+      <c r="M11" s="66" t="s">
+        <v>521</v>
+      </c>
+      <c r="N11" s="68" t="s">
+        <v>529</v>
+      </c>
+      <c r="O11" s="66">
+        <v>130</v>
+      </c>
+      <c r="P11" s="66">
+        <v>160</v>
+      </c>
+      <c r="Q11" s="66">
+        <v>200</v>
+      </c>
+      <c r="R11" s="66">
+        <v>200</v>
+      </c>
+      <c r="S11" s="66">
+        <v>215</v>
+      </c>
+      <c r="T11" s="66">
+        <v>215</v>
+      </c>
+      <c r="U11" s="66">
+        <v>18</v>
+      </c>
+      <c r="V11" s="66">
+        <v>40</v>
+      </c>
+      <c r="W11" s="66">
+        <v>70</v>
+      </c>
+      <c r="X11" s="66">
+        <v>46</v>
+      </c>
+      <c r="Y11" s="66">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="2:25" s="62" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="B12" s="60" t="s">
+        <v>530</v>
+      </c>
+      <c r="C12" s="60" t="s">
+        <v>494</v>
+      </c>
+      <c r="D12" s="66">
+        <v>4.5</v>
+      </c>
+      <c r="E12" s="66">
+        <v>4.8</v>
+      </c>
+      <c r="F12" s="66" t="s">
+        <v>531</v>
+      </c>
+      <c r="G12" s="67"/>
+      <c r="H12" s="66" t="s">
+        <v>532</v>
+      </c>
+      <c r="I12" s="66" t="s">
+        <v>533</v>
+      </c>
+      <c r="J12" s="67"/>
+      <c r="K12" s="67"/>
+      <c r="L12" s="67"/>
+      <c r="M12" s="66" t="s">
+        <v>521</v>
+      </c>
+      <c r="N12" s="68" t="s">
+        <v>522</v>
+      </c>
+      <c r="O12" s="66">
+        <v>130</v>
+      </c>
+      <c r="P12" s="67"/>
+      <c r="Q12" s="66">
+        <v>200</v>
+      </c>
+      <c r="R12" s="67"/>
+      <c r="S12" s="66">
+        <v>215</v>
+      </c>
+      <c r="T12" s="67"/>
+      <c r="U12" s="66">
+        <v>18</v>
+      </c>
+      <c r="V12" s="66">
+        <v>40</v>
+      </c>
+      <c r="W12" s="66">
+        <v>70</v>
+      </c>
+      <c r="X12" s="66">
+        <v>46</v>
+      </c>
+      <c r="Y12" s="66">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="2:25" s="62" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="B13" s="60" t="s">
+        <v>534</v>
+      </c>
+      <c r="C13" s="60" t="s">
+        <v>535</v>
+      </c>
+      <c r="D13" s="66">
+        <v>2.9</v>
+      </c>
+      <c r="E13" s="66">
+        <v>3.2</v>
+      </c>
+      <c r="F13" s="66" t="s">
+        <v>536</v>
+      </c>
+      <c r="G13" s="67"/>
+      <c r="H13" s="67"/>
+      <c r="I13" s="66" t="s">
+        <v>537</v>
+      </c>
+      <c r="J13" s="67"/>
+      <c r="K13" s="66" t="s">
+        <v>538</v>
+      </c>
+      <c r="L13" s="67"/>
+      <c r="M13" s="66" t="s">
+        <v>539</v>
+      </c>
+      <c r="N13" s="68" t="s">
+        <v>540</v>
+      </c>
+      <c r="O13" s="66">
+        <v>120</v>
+      </c>
+      <c r="P13" s="66">
+        <v>160</v>
+      </c>
+      <c r="Q13" s="66">
+        <v>200</v>
+      </c>
+      <c r="R13" s="66">
+        <v>200</v>
+      </c>
+      <c r="S13" s="66">
+        <v>215</v>
+      </c>
+      <c r="T13" s="66">
+        <v>215</v>
+      </c>
+      <c r="U13" s="66">
+        <v>17</v>
+      </c>
+      <c r="V13" s="66">
+        <v>30</v>
+      </c>
+      <c r="W13" s="66">
+        <v>60</v>
+      </c>
+      <c r="X13" s="66">
+        <v>35</v>
+      </c>
+      <c r="Y13" s="66">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="2:25" s="72" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="B14" s="69" t="s">
+        <v>541</v>
+      </c>
+      <c r="C14" s="69" t="s">
+        <v>535</v>
+      </c>
+      <c r="D14" s="70">
+        <v>2.7</v>
+      </c>
+      <c r="E14" s="70">
+        <v>3</v>
+      </c>
+      <c r="F14" s="70">
+        <v>2.5</v>
+      </c>
+      <c r="G14" s="70"/>
+      <c r="H14" s="70"/>
+      <c r="I14" s="70" t="s">
+        <v>542</v>
+      </c>
+      <c r="J14" s="70"/>
+      <c r="K14" s="70"/>
+      <c r="L14" s="70"/>
+      <c r="M14" s="66" t="s">
+        <v>543</v>
+      </c>
+      <c r="N14" s="71" t="s">
+        <v>544</v>
+      </c>
+      <c r="O14" s="70">
+        <v>144</v>
+      </c>
+      <c r="P14" s="70">
+        <v>150</v>
+      </c>
+      <c r="Q14" s="70">
+        <v>240</v>
+      </c>
+      <c r="R14" s="70">
+        <v>200</v>
+      </c>
+      <c r="S14" s="70">
+        <v>270</v>
+      </c>
+      <c r="T14" s="66" t="s">
+        <v>545</v>
+      </c>
+      <c r="U14" s="70">
+        <v>15</v>
+      </c>
+      <c r="V14" s="70">
+        <v>40</v>
+      </c>
+      <c r="W14" s="70">
+        <v>60</v>
+      </c>
+      <c r="X14" s="70">
+        <v>35</v>
+      </c>
+      <c r="Y14" s="70">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="2:25" s="62" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="88" t="s">
+        <v>546</v>
+      </c>
+      <c r="C15" s="88"/>
+      <c r="D15" s="88"/>
+      <c r="E15" s="88"/>
+      <c r="F15" s="88"/>
+      <c r="G15" s="88"/>
+      <c r="H15" s="88"/>
+      <c r="I15" s="88"/>
+      <c r="J15" s="88"/>
+      <c r="K15" s="88"/>
+      <c r="L15" s="88"/>
+      <c r="M15" s="88"/>
+      <c r="N15" s="88"/>
+    </row>
+    <row r="16" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B16" s="77" t="s">
+        <v>547</v>
+      </c>
+      <c r="C16" s="77"/>
+      <c r="D16" s="77"/>
+      <c r="E16" s="77"/>
+      <c r="F16" s="77"/>
+      <c r="G16" s="77"/>
+      <c r="H16" s="77"/>
+      <c r="I16" s="77"/>
+      <c r="J16" s="77"/>
+      <c r="K16" s="77"/>
+      <c r="L16" s="77"/>
+      <c r="M16" s="77"/>
+      <c r="N16" s="77"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="G2:L2"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="Q2:R2"/>
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="B16:N16"/>
+    <mergeCell ref="B15:N15"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
BOM Calculation page adjustments2
</commit_message>
<xml_diff>
--- a/data/Sources.xlsx
+++ b/data/Sources.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pfnonwovens-my.sharepoint.com/personal/mfischer_pfnonwovens_com/Documents/Desktop/mini-erp-node/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="8_{66A118C3-EF46-4704-A6DB-C24509B266D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37174538-E850-4CAF-AE52-6F19ADE6659F}"/>
+  <xr:revisionPtr revIDLastSave="92" documentId="8_{66A118C3-EF46-4704-A6DB-C24509B266D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10BA9B79-48D8-4C88-AC7C-08D74E033D02}"/>
   <bookViews>
     <workbookView xWindow="30105" yWindow="-7095" windowWidth="22575" windowHeight="12585" activeTab="2" xr2:uid="{B924FA10-533B-4C07-A917-FCB6B882FB42}"/>
   </bookViews>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="548">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="538">
   <si>
     <t>SB1</t>
   </si>
@@ -1507,9 +1507,6 @@
   </si>
   <si>
     <t>-</t>
-  </si>
-  <si>
-    <t>L01</t>
   </si>
   <si>
     <t>10gsm 3,10m  130gsm 3,2m</t>
@@ -1536,9 +1533,6 @@
     </r>
   </si>
   <si>
-    <t>L02</t>
-  </si>
-  <si>
     <t xml:space="preserve">12gsm 3,05 m 100gsm 3,20 m </t>
   </si>
   <si>
@@ -1552,9 +1546,6 @@
   </si>
   <si>
     <t>75 (70mmrole)</t>
-  </si>
-  <si>
-    <t>L03</t>
   </si>
   <si>
     <t xml:space="preserve">10gsm 2,90m            80gsm 3,20m </t>
@@ -1587,9 +1578,6 @@
     </r>
   </si>
   <si>
-    <t>L05</t>
-  </si>
-  <si>
     <t>SSMMS</t>
   </si>
   <si>
@@ -1611,9 +1599,6 @@
     <t>580m/min          12gsm</t>
   </si>
   <si>
-    <t>L07</t>
-  </si>
-  <si>
     <t>SSS</t>
   </si>
   <si>
@@ -1635,9 +1620,6 @@
     <t>580 m/min 12gsm</t>
   </si>
   <si>
-    <t>L08</t>
-  </si>
-  <si>
     <t>12gsm - 3,696    25gsm - 4,060</t>
   </si>
   <si>
@@ -1653,9 +1635,6 @@
     <t>755m/min            12gsm</t>
   </si>
   <si>
-    <t>L09</t>
-  </si>
-  <si>
     <t>SSMMMS</t>
   </si>
   <si>
@@ -1680,9 +1659,6 @@
     <t>37 (35funkčních)</t>
   </si>
   <si>
-    <t>L10</t>
-  </si>
-  <si>
     <t>12gsm 4,100m   40g 4,300m</t>
   </si>
   <si>
@@ -1698,9 +1674,6 @@
     <t>1150m/min   7gsm</t>
   </si>
   <si>
-    <t>EL01</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 25gsm  4,080m       12gsm 3,642m</t>
   </si>
   <si>
@@ -1710,9 +1683,6 @@
     <t>15gsm 4,004m   10gsm 3,836m</t>
   </si>
   <si>
-    <t>L11</t>
-  </si>
-  <si>
     <t>SMMS</t>
   </si>
   <si>
@@ -1731,9 +1701,6 @@
     <t>600m/min 8gsm</t>
   </si>
   <si>
-    <t>L12*</t>
-  </si>
-  <si>
     <t>7gsm 2,160m</t>
   </si>
   <si>
@@ -1750,6 +1717,9 @@
   </si>
   <si>
     <t>* u této linky je HAK a HAF kde proudí horký vzduch kolem 150 - 170 °C</t>
+  </si>
+  <si>
+    <t>CZ12*</t>
   </si>
 </sst>
 </file>
@@ -7755,7 +7725,7 @@
   <sheetFormatPr defaultColWidth="6.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="1.109375" style="73" customWidth="1"/>
-    <col min="2" max="2" width="5" style="73" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" style="73" customWidth="1"/>
     <col min="3" max="3" width="10" style="73" customWidth="1"/>
     <col min="4" max="4" width="7" style="73" customWidth="1"/>
     <col min="5" max="5" width="13.109375" style="73" customWidth="1"/>
@@ -7896,7 +7866,7 @@
     </row>
     <row r="4" spans="2:25" s="62" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
       <c r="B4" s="63" t="s">
-        <v>475</v>
+        <v>22</v>
       </c>
       <c r="C4" s="63" t="s">
         <v>26</v>
@@ -7908,7 +7878,7 @@
         <v>3.55</v>
       </c>
       <c r="F4" s="63" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="G4" s="64"/>
       <c r="H4" s="64"/>
@@ -7917,10 +7887,10 @@
       <c r="K4" s="64"/>
       <c r="L4" s="64"/>
       <c r="M4" s="63" t="s">
+        <v>476</v>
+      </c>
+      <c r="N4" s="63" t="s">
         <v>477</v>
-      </c>
-      <c r="N4" s="63" t="s">
-        <v>478</v>
       </c>
       <c r="O4" s="63">
         <v>71</v>
@@ -7941,12 +7911,12 @@
         <v>24</v>
       </c>
       <c r="Y4" s="63" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="5" spans="2:25" s="62" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="B5" s="63" t="s">
-        <v>480</v>
+        <v>34</v>
       </c>
       <c r="C5" s="63" t="s">
         <v>59</v>
@@ -7958,21 +7928,21 @@
         <v>3.6</v>
       </c>
       <c r="F5" s="63" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="G5" s="64"/>
       <c r="H5" s="64"/>
       <c r="I5" s="63" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="J5" s="64"/>
       <c r="K5" s="64"/>
       <c r="L5" s="64"/>
       <c r="M5" s="63" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="N5" s="63" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="O5" s="63">
         <v>97</v>
@@ -7999,12 +7969,12 @@
         <v>40</v>
       </c>
       <c r="Y5" s="65" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="6" spans="2:25" s="62" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
       <c r="B6" s="63" t="s">
-        <v>486</v>
+        <v>45</v>
       </c>
       <c r="C6" s="63" t="s">
         <v>59</v>
@@ -8016,23 +7986,23 @@
         <v>3.8</v>
       </c>
       <c r="F6" s="63" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="G6" s="63" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="H6" s="64"/>
       <c r="I6" s="63" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="J6" s="64"/>
       <c r="K6" s="64"/>
       <c r="L6" s="64"/>
       <c r="M6" s="63" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="N6" s="63" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="O6" s="63">
         <v>135</v>
@@ -8059,15 +8029,15 @@
         <v>38</v>
       </c>
       <c r="Y6" s="63" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
     </row>
     <row r="7" spans="2:25" s="62" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
       <c r="B7" s="60" t="s">
-        <v>493</v>
+        <v>55</v>
       </c>
       <c r="C7" s="60" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="D7" s="66">
         <v>3.5</v>
@@ -8076,25 +8046,25 @@
         <v>3.8</v>
       </c>
       <c r="F7" s="66" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
       <c r="G7" s="67"/>
       <c r="H7" s="67"/>
       <c r="I7" s="66" t="s">
-        <v>496</v>
+        <v>492</v>
       </c>
       <c r="J7" s="67"/>
       <c r="K7" s="66" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="L7" s="66" t="s">
-        <v>498</v>
+        <v>494</v>
       </c>
       <c r="M7" s="66" t="s">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="N7" s="66" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="O7" s="66">
         <v>135</v>
@@ -8132,10 +8102,10 @@
     </row>
     <row r="8" spans="2:25" s="62" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
       <c r="B8" s="60" t="s">
-        <v>501</v>
+        <v>66</v>
       </c>
       <c r="C8" s="60" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="D8" s="66">
         <v>3.5</v>
@@ -8144,25 +8114,25 @@
         <v>3.8</v>
       </c>
       <c r="F8" s="66" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="G8" s="66" t="s">
-        <v>504</v>
+        <v>499</v>
       </c>
       <c r="H8" s="67"/>
       <c r="I8" s="67"/>
       <c r="J8" s="67"/>
       <c r="K8" s="66" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="L8" s="66" t="s">
-        <v>506</v>
+        <v>501</v>
       </c>
       <c r="M8" s="66" t="s">
-        <v>507</v>
+        <v>502</v>
       </c>
       <c r="N8" s="66" t="s">
-        <v>508</v>
+        <v>503</v>
       </c>
       <c r="O8" s="66">
         <v>140</v>
@@ -8194,10 +8164,10 @@
     </row>
     <row r="9" spans="2:25" s="62" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="B9" s="60" t="s">
-        <v>509</v>
+        <v>74</v>
       </c>
       <c r="C9" s="60" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="D9" s="66">
         <v>4.5</v>
@@ -8206,23 +8176,23 @@
         <v>4.8</v>
       </c>
       <c r="F9" s="66" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="G9" s="66" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="H9" s="66" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="I9" s="67"/>
       <c r="J9" s="67"/>
       <c r="K9" s="67"/>
       <c r="L9" s="67"/>
       <c r="M9" s="66" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="N9" s="66" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="O9" s="66">
         <v>160</v>
@@ -8248,10 +8218,10 @@
     </row>
     <row r="10" spans="2:25" s="62" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="B10" s="60" t="s">
-        <v>515</v>
+        <v>80</v>
       </c>
       <c r="C10" s="60" t="s">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="D10" s="66">
         <v>3.5</v>
@@ -8260,25 +8230,25 @@
         <v>3.8</v>
       </c>
       <c r="F10" s="66" t="s">
-        <v>517</v>
+        <v>510</v>
       </c>
       <c r="G10" s="66" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="H10" s="67"/>
       <c r="I10" s="66" t="s">
-        <v>519</v>
+        <v>512</v>
       </c>
       <c r="J10" s="66" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="K10" s="67"/>
       <c r="L10" s="67"/>
       <c r="M10" s="66" t="s">
-        <v>521</v>
+        <v>514</v>
       </c>
       <c r="N10" s="68" t="s">
-        <v>522</v>
+        <v>515</v>
       </c>
       <c r="O10" s="66">
         <v>130</v>
@@ -8302,7 +8272,7 @@
         <v>70</v>
       </c>
       <c r="X10" s="66" t="s">
-        <v>523</v>
+        <v>516</v>
       </c>
       <c r="Y10" s="66">
         <v>55</v>
@@ -8310,10 +8280,10 @@
     </row>
     <row r="11" spans="2:25" s="62" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="B11" s="60" t="s">
-        <v>524</v>
+        <v>88</v>
       </c>
       <c r="C11" s="60" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="D11" s="66">
         <v>4.7</v>
@@ -8322,25 +8292,25 @@
         <v>5</v>
       </c>
       <c r="F11" s="66" t="s">
-        <v>525</v>
+        <v>517</v>
       </c>
       <c r="G11" s="67"/>
       <c r="H11" s="67"/>
       <c r="I11" s="66" t="s">
-        <v>526</v>
+        <v>518</v>
       </c>
       <c r="J11" s="67"/>
       <c r="K11" s="66" t="s">
-        <v>527</v>
+        <v>519</v>
       </c>
       <c r="L11" s="66" t="s">
-        <v>528</v>
+        <v>520</v>
       </c>
       <c r="M11" s="66" t="s">
+        <v>514</v>
+      </c>
+      <c r="N11" s="68" t="s">
         <v>521</v>
-      </c>
-      <c r="N11" s="68" t="s">
-        <v>529</v>
       </c>
       <c r="O11" s="66">
         <v>130</v>
@@ -8378,10 +8348,10 @@
     </row>
     <row r="12" spans="2:25" s="62" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
       <c r="B12" s="60" t="s">
-        <v>530</v>
+        <v>107</v>
       </c>
       <c r="C12" s="60" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="D12" s="66">
         <v>4.5</v>
@@ -8390,23 +8360,23 @@
         <v>4.8</v>
       </c>
       <c r="F12" s="66" t="s">
-        <v>531</v>
+        <v>522</v>
       </c>
       <c r="G12" s="67"/>
       <c r="H12" s="66" t="s">
-        <v>532</v>
+        <v>523</v>
       </c>
       <c r="I12" s="66" t="s">
-        <v>533</v>
+        <v>524</v>
       </c>
       <c r="J12" s="67"/>
       <c r="K12" s="67"/>
       <c r="L12" s="67"/>
       <c r="M12" s="66" t="s">
-        <v>521</v>
+        <v>514</v>
       </c>
       <c r="N12" s="68" t="s">
-        <v>522</v>
+        <v>515</v>
       </c>
       <c r="O12" s="66">
         <v>130</v>
@@ -8438,10 +8408,10 @@
     </row>
     <row r="13" spans="2:25" s="62" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
       <c r="B13" s="60" t="s">
-        <v>534</v>
+        <v>94</v>
       </c>
       <c r="C13" s="60" t="s">
-        <v>535</v>
+        <v>525</v>
       </c>
       <c r="D13" s="66">
         <v>2.9</v>
@@ -8450,23 +8420,23 @@
         <v>3.2</v>
       </c>
       <c r="F13" s="66" t="s">
-        <v>536</v>
+        <v>526</v>
       </c>
       <c r="G13" s="67"/>
       <c r="H13" s="67"/>
       <c r="I13" s="66" t="s">
-        <v>537</v>
+        <v>527</v>
       </c>
       <c r="J13" s="67"/>
       <c r="K13" s="66" t="s">
-        <v>538</v>
+        <v>528</v>
       </c>
       <c r="L13" s="67"/>
       <c r="M13" s="66" t="s">
-        <v>539</v>
+        <v>529</v>
       </c>
       <c r="N13" s="68" t="s">
-        <v>540</v>
+        <v>530</v>
       </c>
       <c r="O13" s="66">
         <v>120</v>
@@ -8503,11 +8473,11 @@
       </c>
     </row>
     <row r="14" spans="2:25" s="72" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B14" s="69" t="s">
-        <v>541</v>
+      <c r="B14" s="60" t="s">
+        <v>537</v>
       </c>
       <c r="C14" s="69" t="s">
-        <v>535</v>
+        <v>525</v>
       </c>
       <c r="D14" s="70">
         <v>2.7</v>
@@ -8521,16 +8491,16 @@
       <c r="G14" s="70"/>
       <c r="H14" s="70"/>
       <c r="I14" s="70" t="s">
-        <v>542</v>
+        <v>531</v>
       </c>
       <c r="J14" s="70"/>
       <c r="K14" s="70"/>
       <c r="L14" s="70"/>
       <c r="M14" s="66" t="s">
-        <v>543</v>
+        <v>532</v>
       </c>
       <c r="N14" s="71" t="s">
-        <v>544</v>
+        <v>533</v>
       </c>
       <c r="O14" s="70">
         <v>144</v>
@@ -8548,7 +8518,7 @@
         <v>270</v>
       </c>
       <c r="T14" s="66" t="s">
-        <v>545</v>
+        <v>534</v>
       </c>
       <c r="U14" s="70">
         <v>15</v>
@@ -8568,7 +8538,7 @@
     </row>
     <row r="15" spans="2:25" s="62" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B15" s="88" t="s">
-        <v>546</v>
+        <v>535</v>
       </c>
       <c r="C15" s="88"/>
       <c r="D15" s="88"/>
@@ -8585,7 +8555,7 @@
     </row>
     <row r="16" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B16" s="77" t="s">
-        <v>547</v>
+        <v>536</v>
       </c>
       <c r="C16" s="77"/>
       <c r="D16" s="77"/>

</xml_diff>

<commit_message>
Dodělaný BOM Calc a založena DB
</commit_message>
<xml_diff>
--- a/data/Sources.xlsx
+++ b/data/Sources.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pfnonwovens-my.sharepoint.com/personal/mfischer_pfnonwovens_com/Documents/Desktop/mini-erp-node/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="92" documentId="8_{66A118C3-EF46-4704-A6DB-C24509B266D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10BA9B79-48D8-4C88-AC7C-08D74E033D02}"/>
+  <xr:revisionPtr revIDLastSave="117" documentId="8_{66A118C3-EF46-4704-A6DB-C24509B266D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABB5D6B0-D3E2-4748-BB1A-EF21EDF2D517}"/>
   <bookViews>
-    <workbookView xWindow="30105" yWindow="-7095" windowWidth="22575" windowHeight="12585" activeTab="2" xr2:uid="{B924FA10-533B-4C07-A917-FCB6B882FB42}"/>
+    <workbookView xWindow="28680" yWindow="-11055" windowWidth="29040" windowHeight="17520" xr2:uid="{B924FA10-533B-4C07-A917-FCB6B882FB42}"/>
   </bookViews>
   <sheets>
     <sheet name="Lists" sheetId="1" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="543">
   <si>
     <t>SB1</t>
   </si>
@@ -195,9 +195,6 @@
     <t>Agrimpex</t>
   </si>
   <si>
-    <t>hygiene</t>
-  </si>
-  <si>
     <t>Mono</t>
   </si>
   <si>
@@ -258,9 +255,6 @@
     <t>Attends</t>
   </si>
   <si>
-    <t>technical</t>
-  </si>
-  <si>
     <t>SMS</t>
   </si>
   <si>
@@ -1449,12 +1443,6 @@
     <t>Šířka trysek    (m)</t>
   </si>
   <si>
-    <t>Šířka sítového pásu                 ( m )</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Využitelná šířka NT        **                                                                                                                                                          min / max                                                                                    </t>
-  </si>
-  <si>
     <t>Min. rychlost pásu / max. gsm</t>
   </si>
   <si>
@@ -1480,9 +1468,6 @@
   </si>
   <si>
     <t>Max. počet nožů</t>
-  </si>
-  <si>
-    <t>Min. šířka nožů           ( mm )</t>
   </si>
   <si>
     <t>Mono G1</t>
@@ -1720,6 +1705,37 @@
   </si>
   <si>
     <t>CZ12*</t>
+  </si>
+  <si>
+    <t>Min. šířka nožů (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Využitelná šířka NT **
+min / max                                                                                    </t>
+  </si>
+  <si>
+    <t>Šířka sítového pásu (m)</t>
+  </si>
+  <si>
+    <t>technical - general</t>
+  </si>
+  <si>
+    <t>technical - roofing</t>
+  </si>
+  <si>
+    <t>technical - filtration</t>
+  </si>
+  <si>
+    <t>hygiene - babycare</t>
+  </si>
+  <si>
+    <t>hygiene - femcare</t>
+  </si>
+  <si>
+    <t>hygiene - general</t>
+  </si>
+  <si>
+    <t>homecare</t>
   </si>
 </sst>
 </file>
@@ -2235,7 +2251,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2479,6 +2495,23 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="4" fontId="10" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="10" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2497,23 +2530,7 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="4" fontId="10" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="10" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4074,96 +4091,96 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{4905E39C-E898-4DCE-8992-EB9DD8BDD77C}" name="Structure" displayName="Structure" ref="K1:K17" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36" headerRowCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{4905E39C-E898-4DCE-8992-EB9DD8BDD77C}" name="Structure" displayName="Structure" ref="K1:K17" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39" headerRowCellStyle="Normální 2">
   <autoFilter ref="K1:K17" xr:uid="{4905E39C-E898-4DCE-8992-EB9DD8BDD77C}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{56A23D9B-6A6F-4753-BE1E-C32EC840E0CC}" name="Structure" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{56A23D9B-6A6F-4753-BE1E-C32EC840E0CC}" name="Structure" dataDxfId="38"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{413D5326-F5B7-47B4-B01A-6CB9BA8E80F3}" name="Main_RM" displayName="Main_RM" ref="L1:L21" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{413D5326-F5B7-47B4-B01A-6CB9BA8E80F3}" name="Main_RM" displayName="Main_RM" ref="L1:L21" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
   <autoFilter ref="L1:L21" xr:uid="{413D5326-F5B7-47B4-B01A-6CB9BA8E80F3}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="L2:L21">
     <sortCondition ref="L2:L22"/>
   </sortState>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{DD8457DA-8491-478C-9906-5FD70BAC1D58}" name="Main RawMat" dataDxfId="32" dataCellStyle="Normální 2"/>
+    <tableColumn id="1" xr3:uid="{DD8457DA-8491-478C-9906-5FD70BAC1D58}" name="Main RawMat" dataDxfId="35" dataCellStyle="Normální 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium25" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{1B04A6F5-7D60-4358-A04F-F7B790D5B889}" name="Bonding" displayName="Bonding" ref="M1:M17" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{1B04A6F5-7D60-4358-A04F-F7B790D5B889}" name="Bonding" displayName="Bonding" ref="M1:M17" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
   <autoFilter ref="M1:M17" xr:uid="{1B04A6F5-7D60-4358-A04F-F7B790D5B889}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{56ECAD42-4F9B-4A07-AFE4-7B55C7D60185}" name="Bonding" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{56ECAD42-4F9B-4A07-AFE4-7B55C7D60185}" name="Bonding" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium24" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FC924A71-2AB7-4534-BAF1-472867F8C212}" name="BICO_ratio" displayName="BICO_ratio" ref="N1:N12" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27" headerRowCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FC924A71-2AB7-4534-BAF1-472867F8C212}" name="BICO_ratio" displayName="BICO_ratio" ref="N1:N12" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30" headerRowCellStyle="Normální 2">
   <autoFilter ref="N1:N12" xr:uid="{FC924A71-2AB7-4534-BAF1-472867F8C212}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N2:N12">
     <sortCondition ref="N3:N12"/>
   </sortState>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{328F5A89-E5FD-4981-8CDC-7C47CB509CD7}" name="BICO_ratio" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{328F5A89-E5FD-4981-8CDC-7C47CB509CD7}" name="BICO_ratio" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{C18F5E1C-F12C-48F7-8C94-ECB150008FB8}" name="Treatment" displayName="Treatment" ref="O1:O14" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{C18F5E1C-F12C-48F7-8C94-ECB150008FB8}" name="Treatment" displayName="Treatment" ref="O1:O14" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
   <autoFilter ref="O1:O14" xr:uid="{C18F5E1C-F12C-48F7-8C94-ECB150008FB8}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{B95087BE-BB18-44FB-AB6B-CE34516E6A4E}" name="Treatment" dataDxfId="23" dataCellStyle="Normální 2"/>
+    <tableColumn id="1" xr3:uid="{B95087BE-BB18-44FB-AB6B-CE34516E6A4E}" name="Treatment" dataDxfId="26" dataCellStyle="Normální 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium25" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{69417235-E692-4566-8941-350F0E308BFA}" name="Color" displayName="Color" ref="P1:P74" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{69417235-E692-4566-8941-350F0E308BFA}" name="Color" displayName="Color" ref="P1:P74" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
   <autoFilter ref="P1:P74" xr:uid="{69417235-E692-4566-8941-350F0E308BFA}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{D6D6BE17-33AB-4EE1-90CD-430533094C81}" name="Color" dataDxfId="20" dataCellStyle="Normální 2"/>
+    <tableColumn id="1" xr3:uid="{D6D6BE17-33AB-4EE1-90CD-430533094C81}" name="Color" dataDxfId="23" dataCellStyle="Normální 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium24" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{8074344A-42F3-4096-BA1F-1011EBCE4F62}" name="Cores" displayName="Cores" ref="Q1:Q6" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{8074344A-42F3-4096-BA1F-1011EBCE4F62}" name="Cores" displayName="Cores" ref="Q1:Q6" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
   <autoFilter ref="Q1:Q6" xr:uid="{8074344A-42F3-4096-BA1F-1011EBCE4F62}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{D8816DF6-A4B5-48B7-95B8-92BAF88C9083}" name="Cores" dataDxfId="17" dataCellStyle="Normální 2"/>
+    <tableColumn id="1" xr3:uid="{D8816DF6-A4B5-48B7-95B8-92BAF88C9083}" name="Cores" dataDxfId="20" dataCellStyle="Normální 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{838775E4-F5E0-431D-9351-D17AE56F19D7}" name="Line" displayName="Line" ref="R1:R17" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{838775E4-F5E0-431D-9351-D17AE56F19D7}" name="Line" displayName="Line" ref="R1:R17" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
   <autoFilter ref="R1:R17" xr:uid="{838775E4-F5E0-431D-9351-D17AE56F19D7}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{8390CAA7-046C-4F7E-8958-FFCCA51C7490}" name="Line" dataDxfId="14" dataCellStyle="Normální 2"/>
+    <tableColumn id="1" xr3:uid="{8390CAA7-046C-4F7E-8958-FFCCA51C7490}" name="Line" dataDxfId="17" dataCellStyle="Normální 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium25" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{CD1B2D88-330C-4AA5-92F9-DC81C83DDD5C}" name="Application" displayName="Application" ref="S1:S20" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{CD1B2D88-330C-4AA5-92F9-DC81C83DDD5C}" name="Application" displayName="Application" ref="S1:S20" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="S1:S20" xr:uid="{CD1B2D88-330C-4AA5-92F9-DC81C83DDD5C}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{07F71864-2ADD-444A-9722-A87171922B3B}" name="Application" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{07F71864-2ADD-444A-9722-A87171922B3B}" name="Application" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium24" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4224,33 +4241,36 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{900597CB-2276-43CA-8635-9ED863BCF790}" name="Segment" displayName="Segment" ref="H1:H7" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45" headerRowCellStyle="Normální 2">
-  <autoFilter ref="H1:H7" xr:uid="{900597CB-2276-43CA-8635-9ED863BCF790}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{900597CB-2276-43CA-8635-9ED863BCF790}" name="Segment" displayName="Segment" ref="H1:H12" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12" headerRowCellStyle="Normální 2">
+  <autoFilter ref="H1:H12" xr:uid="{900597CB-2276-43CA-8635-9ED863BCF790}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="H2:H11">
+    <sortCondition ref="H5:H11"/>
+  </sortState>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{938C3C67-4ACA-4662-9C57-E897A4B22B13}" name="Segment" dataDxfId="44"/>
+    <tableColumn id="1" xr3:uid="{938C3C67-4ACA-4662-9C57-E897A4B22B13}" name="Segment" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{6464D72C-C69A-4112-8424-97766E88D7C7}" name="S_SMS" displayName="S_SMS" ref="I1:I3" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42" headerRowCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{6464D72C-C69A-4112-8424-97766E88D7C7}" name="S_SMS" displayName="S_SMS" ref="I1:I3" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45" headerRowCellStyle="Normální 2">
   <autoFilter ref="I1:I3" xr:uid="{6464D72C-C69A-4112-8424-97766E88D7C7}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{139A78FA-5925-4655-AE99-194FDAFDFE73}" name="S/SMS" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{139A78FA-5925-4655-AE99-194FDAFDFE73}" name="S/SMS" dataDxfId="44"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium25" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{6F590121-595E-4041-9C49-F227887713EB}" name="Mono_Bico" displayName="Mono_Bico" ref="J1:J4" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39" headerRowCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{6F590121-595E-4041-9C49-F227887713EB}" name="Mono_Bico" displayName="Mono_Bico" ref="J1:J4" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42" headerRowCellStyle="Normální 2">
   <autoFilter ref="J1:J4" xr:uid="{6F590121-595E-4041-9C49-F227887713EB}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="J2:J4">
     <sortCondition descending="1" ref="J2:J4"/>
   </sortState>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{49BE5F34-76EF-4FC6-AD85-4A01D164CFDE}" name="Mono/Bico" dataDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{49BE5F34-76EF-4FC6-AD85-4A01D164CFDE}" name="Mono/Bico" dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium24" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4598,46 +4618,46 @@
   <sheetData>
     <row r="1" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="57" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>6</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>7</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="O1" s="4" t="s">
         <v>8</v>
@@ -4649,7 +4669,7 @@
         <v>9</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="S1" s="3" t="s">
         <v>10</v>
@@ -4657,19 +4677,19 @@
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="F2" s="8">
         <v>1</v>
@@ -4684,7 +4704,7 @@
         <v>26</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="K2" s="5" t="s">
         <v>15</v>
@@ -4716,19 +4736,19 @@
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="F3" s="8">
         <v>1</v>
@@ -4740,7 +4760,7 @@
         <v>25</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>27</v>
@@ -4775,19 +4795,19 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="F4" s="8">
         <v>0.99</v>
@@ -4795,279 +4815,285 @@
       <c r="G4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="H4" s="5" t="s">
-        <v>37</v>
+      <c r="H4" s="89" t="s">
+        <v>542</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>14</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="L4" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="M4" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="N4" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="N4" s="5" t="s">
+      <c r="O4" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="P4" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="P4" s="7" t="s">
+      <c r="Q4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="Q4" s="7" t="s">
+      <c r="R4" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="R4" s="7" t="s">
+      <c r="S4" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="S4" s="5" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="F5" s="8">
         <v>1</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H5" s="5" t="s">
+        <v>541</v>
+      </c>
+      <c r="K5" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="K5" s="5" t="s">
+      <c r="L5" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L5" s="7" t="s">
+      <c r="M5" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="N5" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="M5" s="5" t="s">
-        <v>388</v>
-      </c>
-      <c r="N5" s="5" t="s">
+      <c r="O5" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="P5" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="Q5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="Q5" s="7" t="s">
+      <c r="R5" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="R5" s="7" t="s">
+      <c r="S5" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="S5" s="5" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="F6" s="8">
         <v>0.5</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
+      </c>
+      <c r="H6" s="89" t="s">
+        <v>539</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="M6" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="O6" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="N6" s="5" t="s">
+      <c r="P6" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="Q6" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="P6" s="7" t="s">
+      <c r="R6" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="Q6" s="7" t="s">
+      <c r="S6" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="R6" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="S6" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="F7" s="8">
         <v>1</v>
       </c>
       <c r="G7" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="H7" s="89" t="s">
+        <v>540</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="M7" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="H7" s="5" t="s">
-        <v>274</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>431</v>
-      </c>
-      <c r="L7" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="M7" s="5" t="s">
+      <c r="N7" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="O7" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="P7" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="R7" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="P7" s="7" t="s">
+      <c r="S7" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="R7" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="S7" s="5" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="F8" s="8">
         <v>1</v>
       </c>
       <c r="G8" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>441</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="O8" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="K8" s="5" t="s">
-        <v>432</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>443</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>389</v>
-      </c>
-      <c r="N8" s="5" t="s">
+      <c r="P8" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="O8" s="7" t="s">
+      <c r="R8" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="P8" s="7" t="s">
+      <c r="S8" s="5" t="s">
         <v>79</v>
-      </c>
-      <c r="R8" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="S8" s="5" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="F9" s="8">
         <v>0.45</v>
       </c>
       <c r="G9" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>536</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="M9" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="K9" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="L9" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="M9" s="5" t="s">
+      <c r="N9" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="O9" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="N9" s="5" t="s">
+      <c r="P9" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="R9" s="7" t="s">
         <v>86</v>
-      </c>
-      <c r="P9" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="R9" s="7" t="s">
-        <v>88</v>
       </c>
       <c r="S9" s="5" t="s">
         <v>15</v>
@@ -5075,1141 +5101,1150 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="F10" s="8">
         <v>0.94</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>89</v>
+        <v>87</v>
+      </c>
+      <c r="H10" s="89" t="s">
+        <v>538</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="O10" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="P10" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="R10" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="P10" s="7" t="s">
+      <c r="S10" s="5" t="s">
         <v>93</v>
-      </c>
-      <c r="R10" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="S10" s="5" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="F11" s="8">
         <v>0.43</v>
       </c>
       <c r="G11" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="H11" s="89" t="s">
+        <v>537</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="N11" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="O11" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="K11" s="5" t="s">
-        <v>435</v>
-      </c>
-      <c r="L11" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="M11" s="5" t="s">
-        <v>387</v>
-      </c>
-      <c r="N11" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="O11" s="7" t="s">
+      <c r="P11" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="R11" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="P11" s="7" t="s">
+      <c r="S11" s="5" t="s">
         <v>99</v>
-      </c>
-      <c r="R11" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="S11" s="5" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F12" s="8">
         <v>0.5</v>
       </c>
       <c r="G12" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="H12" s="89" t="s">
+        <v>272</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="M12" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="K12" s="5" t="s">
-        <v>436</v>
-      </c>
-      <c r="L12" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="M12" s="5" t="s">
+      <c r="N12" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="O12" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="P12" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="N12" s="7" t="s">
-        <v>274</v>
-      </c>
-      <c r="O12" s="7" t="s">
+      <c r="R12" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="P12" s="7" t="s">
+      <c r="S12" s="5" t="s">
         <v>106</v>
-      </c>
-      <c r="R12" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="S12" s="5" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="F13" s="8">
         <v>0.5</v>
       </c>
       <c r="G13" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="M13" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="K13" s="5" t="s">
-        <v>437</v>
-      </c>
-      <c r="L13" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="M13" s="5" t="s">
+      <c r="O13" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="P13" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="O13" s="7" t="s">
+      <c r="R13" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="P13" s="7" t="s">
+      <c r="S13" s="5" t="s">
         <v>113</v>
-      </c>
-      <c r="R13" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="S13" s="5" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="F14" s="8">
         <v>0.76</v>
       </c>
       <c r="G14" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="M14" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="O14" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="K14" s="5" t="s">
-        <v>438</v>
-      </c>
-      <c r="L14" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="M14" s="5" t="s">
-        <v>444</v>
-      </c>
-      <c r="O14" s="7" t="s">
+      <c r="P14" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="R14" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="P14" s="7" t="s">
+      <c r="S14" s="5" t="s">
         <v>119</v>
-      </c>
-      <c r="R14" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="S14" s="5" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="F15" s="8">
         <v>0.96</v>
       </c>
       <c r="G15" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="M15" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="P15" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="K15" s="5" t="s">
-        <v>439</v>
-      </c>
-      <c r="L15" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="M15" s="5" t="s">
-        <v>445</v>
-      </c>
-      <c r="P15" s="7" t="s">
-        <v>124</v>
-      </c>
       <c r="R15" s="7" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="S15" s="5" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="F16" s="8">
         <v>0.19</v>
       </c>
       <c r="G16" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="M16" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="P16" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="K16" s="5" t="s">
-        <v>440</v>
-      </c>
-      <c r="L16" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="M16" s="5" t="s">
-        <v>446</v>
-      </c>
-      <c r="P16" s="7" t="s">
-        <v>128</v>
-      </c>
       <c r="R16" s="7" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="S16" s="5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="F17" s="8">
         <v>0.2</v>
       </c>
       <c r="G17" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="M17" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="P17" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="K17" s="5" t="s">
-        <v>441</v>
-      </c>
-      <c r="L17" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="M17" s="5" t="s">
+      <c r="R17" s="7" t="s">
         <v>447</v>
       </c>
-      <c r="P17" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="R17" s="7" t="s">
-        <v>449</v>
-      </c>
       <c r="S17" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="F18" s="8">
         <v>0.6</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="M18" s="58"/>
       <c r="P18" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="R18" s="7"/>
       <c r="S18" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="F19" s="8">
         <v>1</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="M19" s="58"/>
       <c r="P19" s="7" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="R19" s="7"/>
       <c r="S19" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="F20" s="8">
         <v>0.03</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="M20" s="58"/>
       <c r="P20" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="R20" s="7"/>
       <c r="S20" s="5" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="21" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="F21" s="8">
         <v>0.7</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="M21" s="58"/>
       <c r="P21" s="7" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="R21" s="7"/>
     </row>
     <row r="22" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="L22" s="58"/>
       <c r="M22" s="58"/>
       <c r="P22" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="R22" s="7"/>
     </row>
     <row r="23" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="5" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="L23" s="58"/>
       <c r="M23" s="58"/>
       <c r="P23" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="R23" s="7"/>
     </row>
     <row r="24" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L24" s="58"/>
       <c r="M24" s="58"/>
       <c r="P24" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="R24" s="7"/>
     </row>
     <row r="25" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="5" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="L25" s="58"/>
       <c r="M25" s="58"/>
       <c r="P25" s="7" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="R25" s="7"/>
     </row>
     <row r="26" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="5" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="L26" s="58"/>
       <c r="M26" s="58"/>
       <c r="P26" s="7" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="R26" s="7"/>
     </row>
     <row r="27" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="L27" s="58"/>
       <c r="P27" s="7" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="R27" s="7"/>
     </row>
     <row r="28" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="5" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="L28" s="58"/>
       <c r="P28" s="7" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="R28" s="7"/>
     </row>
     <row r="29" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="5" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="L29" s="58"/>
       <c r="P29" s="7" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="R29" s="7"/>
     </row>
     <row r="30" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="5" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="L30" s="58"/>
       <c r="P30" s="7" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="R30" s="7"/>
     </row>
     <row r="31" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="5" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="L31" s="58"/>
       <c r="P31" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R31" s="7"/>
     </row>
     <row r="32" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C32" s="5" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="5" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="L32" s="58"/>
       <c r="P32" s="7" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="R32" s="7"/>
     </row>
     <row r="33" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C33" s="5" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="5" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="L33" s="58"/>
       <c r="P33" s="7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="R33" s="7"/>
     </row>
     <row r="34" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C34" s="5" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="5" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="L34" s="58"/>
       <c r="P34" s="7" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="R34" s="7"/>
     </row>
     <row r="35" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C35" s="5" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="L35" s="58"/>
       <c r="P35" s="7" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="R35" s="7"/>
     </row>
     <row r="36" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C36" s="5" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="L36" s="58"/>
       <c r="P36" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="R36" s="7"/>
     </row>
     <row r="37" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C37" s="5" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="F37" s="6"/>
       <c r="G37" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="L37" s="58"/>
       <c r="P37" s="7" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="R37" s="7"/>
     </row>
     <row r="38" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C38" s="5" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="L38" s="58"/>
       <c r="P38" s="7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="R38" s="7"/>
     </row>
     <row r="39" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C39" s="5" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="F39" s="6"/>
       <c r="G39" s="5" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="L39" s="58"/>
       <c r="P39" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="R39" s="7"/>
     </row>
     <row r="40" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C40" s="5" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="L40" s="58"/>
       <c r="P40" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="R40" s="7"/>
     </row>
     <row r="41" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C41" s="5" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="L41" s="58"/>
       <c r="P41" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="R41" s="7"/>
     </row>
     <row r="42" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C42" s="5" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F42" s="6"/>
       <c r="G42" s="5" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="L42" s="7"/>
       <c r="P42" s="7" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="R42" s="7"/>
     </row>
     <row r="43" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C43" s="5" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F43" s="6"/>
       <c r="G43" s="5" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="L43" s="7"/>
       <c r="P43" s="7" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="R43" s="7"/>
     </row>
     <row r="44" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C44" s="5" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F44" s="6"/>
       <c r="G44" s="5" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="L44" s="7"/>
       <c r="P44" s="7" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="R44" s="7"/>
     </row>
     <row r="45" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C45" s="5" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F45" s="6"/>
       <c r="G45" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="L45" s="7"/>
       <c r="P45" s="7" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="R45" s="7"/>
     </row>
     <row r="46" spans="3:18" x14ac:dyDescent="0.2">
       <c r="F46" s="6"/>
       <c r="G46" s="5" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="L46" s="7"/>
       <c r="P46" s="7" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="R46" s="7"/>
     </row>
     <row r="47" spans="3:18" x14ac:dyDescent="0.2">
       <c r="F47" s="6"/>
       <c r="G47" s="5" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="L47" s="7"/>
       <c r="P47" s="7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="R47" s="7"/>
     </row>
     <row r="48" spans="3:18" x14ac:dyDescent="0.2">
       <c r="F48" s="6"/>
       <c r="G48" s="5" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="L48" s="7"/>
       <c r="P48" s="7" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="R48" s="7"/>
     </row>
     <row r="49" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F49" s="6"/>
       <c r="G49" s="5" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="L49" s="7"/>
       <c r="P49" s="7" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="R49" s="7"/>
     </row>
     <row r="50" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F50" s="6"/>
       <c r="G50" s="5" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L50" s="7"/>
       <c r="P50" s="7" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="R50" s="7"/>
     </row>
     <row r="51" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F51" s="6"/>
       <c r="G51" s="5" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L51" s="7"/>
       <c r="P51" s="7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="R51" s="7"/>
     </row>
     <row r="52" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F52" s="6"/>
       <c r="G52" s="5" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L52" s="7"/>
       <c r="P52" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="R52" s="7"/>
     </row>
     <row r="53" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F53" s="6"/>
       <c r="G53" s="5" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="L53" s="7"/>
       <c r="P53" s="7" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="R53" s="7"/>
     </row>
     <row r="54" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F54" s="6"/>
       <c r="G54" s="5" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="L54" s="7"/>
       <c r="P54" s="7" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="R54" s="7"/>
     </row>
     <row r="55" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F55" s="6"/>
       <c r="G55" s="5" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="L55" s="7"/>
       <c r="P55" s="7" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="R55" s="7"/>
     </row>
     <row r="56" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F56" s="6"/>
       <c r="G56" s="5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="L56" s="7"/>
       <c r="P56" s="7" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="R56" s="7"/>
     </row>
     <row r="57" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F57" s="6"/>
       <c r="G57" s="5" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L57" s="7"/>
       <c r="P57" s="7" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="R57" s="7"/>
     </row>
     <row r="58" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F58" s="6"/>
       <c r="G58" s="5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="L58" s="7"/>
       <c r="P58" s="7" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="R58" s="7"/>
     </row>
     <row r="59" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F59" s="6"/>
       <c r="G59" s="5" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="L59" s="7"/>
       <c r="P59" s="7" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="R59" s="7"/>
     </row>
     <row r="60" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F60" s="6"/>
       <c r="G60" s="5" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="L60" s="7"/>
       <c r="P60" s="7" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="R60" s="7"/>
     </row>
     <row r="61" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F61" s="6"/>
       <c r="G61" s="5" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="L61" s="7"/>
       <c r="P61" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="R61" s="7"/>
     </row>
     <row r="62" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F62" s="6"/>
       <c r="G62" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="L62" s="7"/>
       <c r="P62" s="7" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="R62" s="7"/>
     </row>
     <row r="63" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F63" s="6"/>
       <c r="G63" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="L63" s="7"/>
       <c r="P63" s="7" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="R63" s="7"/>
     </row>
     <row r="64" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F64" s="6"/>
       <c r="G64" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="L64" s="7"/>
       <c r="P64" s="7" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="R64" s="7"/>
     </row>
     <row r="65" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F65" s="6"/>
       <c r="G65" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="L65" s="7"/>
       <c r="P65" s="7" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="R65" s="7"/>
     </row>
     <row r="66" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F66" s="6"/>
       <c r="G66" s="5" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L66" s="7"/>
       <c r="P66" s="7" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="R66" s="7"/>
     </row>
     <row r="67" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F67" s="6"/>
       <c r="G67" s="5" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="L67" s="7"/>
       <c r="P67" s="7" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="R67" s="7"/>
     </row>
     <row r="68" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F68" s="6"/>
       <c r="G68" s="5" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="L68" s="7"/>
       <c r="P68" s="7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="R68" s="7"/>
     </row>
     <row r="69" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F69" s="6"/>
       <c r="G69" s="5" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="L69" s="7"/>
       <c r="P69" s="7" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="R69" s="7"/>
     </row>
     <row r="70" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F70" s="6"/>
       <c r="G70" s="5" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="L70" s="7"/>
       <c r="P70" s="7" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="R70" s="7"/>
     </row>
     <row r="71" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F71" s="6"/>
       <c r="G71" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="L71" s="7"/>
       <c r="P71" s="7" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="R71" s="7"/>
     </row>
     <row r="72" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F72" s="6"/>
       <c r="G72" s="5" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L72" s="7"/>
       <c r="P72" s="7" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="R72" s="7"/>
     </row>
     <row r="73" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F73" s="6"/>
       <c r="G73" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="L73" s="7"/>
       <c r="P73" s="7" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="R73" s="7"/>
     </row>
     <row r="74" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F74" s="6"/>
       <c r="G74" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="L74" s="7"/>
       <c r="P74" s="7" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="R74" s="7"/>
     </row>
     <row r="75" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F75" s="6"/>
       <c r="G75" s="5" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="L75" s="7"/>
       <c r="R75" s="7"/>
@@ -6217,7 +6252,7 @@
     <row r="76" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F76" s="6"/>
       <c r="G76" s="5" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="L76" s="7"/>
       <c r="R76" s="7"/>
@@ -6225,7 +6260,7 @@
     <row r="77" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F77" s="6"/>
       <c r="G77" s="5" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="L77" s="7"/>
       <c r="R77" s="7"/>
@@ -6233,7 +6268,7 @@
     <row r="78" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F78" s="6"/>
       <c r="G78" s="5" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="L78" s="7"/>
       <c r="R78" s="7"/>
@@ -6241,7 +6276,7 @@
     <row r="79" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F79" s="6"/>
       <c r="G79" s="5" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="L79" s="7"/>
       <c r="R79" s="7"/>
@@ -6249,7 +6284,7 @@
     <row r="80" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F80" s="6"/>
       <c r="G80" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="L80" s="7"/>
       <c r="R80" s="7"/>
@@ -6257,7 +6292,7 @@
     <row r="81" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F81" s="6"/>
       <c r="G81" s="5" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="L81" s="7"/>
       <c r="R81" s="7"/>
@@ -6265,7 +6300,7 @@
     <row r="82" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F82" s="6"/>
       <c r="G82" s="5" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="L82" s="7"/>
       <c r="R82" s="7"/>
@@ -6273,7 +6308,7 @@
     <row r="83" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F83" s="6"/>
       <c r="G83" s="5" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="L83" s="7"/>
       <c r="R83" s="7"/>
@@ -6281,7 +6316,7 @@
     <row r="84" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F84" s="6"/>
       <c r="G84" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="L84" s="7"/>
       <c r="R84" s="7"/>
@@ -6289,7 +6324,7 @@
     <row r="85" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F85" s="6"/>
       <c r="G85" s="5" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="L85" s="7"/>
       <c r="R85" s="7"/>
@@ -6297,7 +6332,7 @@
     <row r="86" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F86" s="6"/>
       <c r="G86" s="5" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="L86" s="7"/>
       <c r="R86" s="7"/>
@@ -6305,7 +6340,7 @@
     <row r="87" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F87" s="6"/>
       <c r="G87" s="5" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="L87" s="7"/>
       <c r="R87" s="7"/>
@@ -6397,7 +6432,7 @@
     <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" s="9"/>
       <c r="B1" s="10" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C1" s="9"/>
       <c r="D1" s="9"/>
@@ -6432,7 +6467,7 @@
         <v>1000</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="E2" s="9"/>
       <c r="F2" s="9"/>
@@ -6461,14 +6496,14 @@
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" s="10"/>
       <c r="B3" s="10"/>
-      <c r="C3" s="78" t="s">
-        <v>266</v>
-      </c>
-      <c r="D3" s="79"/>
-      <c r="E3" s="78" t="s">
-        <v>266</v>
-      </c>
-      <c r="F3" s="79"/>
+      <c r="C3" s="83" t="s">
+        <v>264</v>
+      </c>
+      <c r="D3" s="84"/>
+      <c r="E3" s="83" t="s">
+        <v>264</v>
+      </c>
+      <c r="F3" s="84"/>
       <c r="G3" s="14" t="s">
         <v>13</v>
       </c>
@@ -6481,14 +6516,14 @@
       <c r="J3" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="K3" s="80" t="s">
-        <v>266</v>
-      </c>
-      <c r="L3" s="81"/>
-      <c r="M3" s="78" t="s">
-        <v>266</v>
-      </c>
-      <c r="N3" s="79"/>
+      <c r="K3" s="85" t="s">
+        <v>264</v>
+      </c>
+      <c r="L3" s="86"/>
+      <c r="M3" s="83" t="s">
+        <v>264</v>
+      </c>
+      <c r="N3" s="84"/>
       <c r="O3" s="9"/>
       <c r="P3" s="9"/>
       <c r="Q3" s="13"/>
@@ -6505,37 +6540,37 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
+        <v>391</v>
+      </c>
+      <c r="B4" s="16"/>
+      <c r="C4" s="87" t="s">
+        <v>392</v>
+      </c>
+      <c r="D4" s="88"/>
+      <c r="E4" s="87" t="s">
         <v>393</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="82" t="s">
+      <c r="F4" s="88"/>
+      <c r="G4" s="17" t="s">
         <v>394</v>
       </c>
-      <c r="D4" s="83"/>
-      <c r="E4" s="82" t="s">
+      <c r="H4" s="15" t="s">
         <v>395</v>
       </c>
-      <c r="F4" s="83"/>
-      <c r="G4" s="17" t="s">
+      <c r="I4" s="17" t="s">
         <v>396</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="J4" s="15" t="s">
         <v>397</v>
       </c>
-      <c r="I4" s="17" t="s">
+      <c r="K4" s="87" t="s">
         <v>398</v>
       </c>
-      <c r="J4" s="15" t="s">
+      <c r="L4" s="88"/>
+      <c r="M4" s="87" t="s">
         <v>399</v>
       </c>
-      <c r="K4" s="82" t="s">
-        <v>400</v>
-      </c>
-      <c r="L4" s="83"/>
-      <c r="M4" s="82" t="s">
-        <v>401</v>
-      </c>
-      <c r="N4" s="83"/>
+      <c r="N4" s="88"/>
       <c r="O4" s="9"/>
       <c r="P4" s="9"/>
       <c r="Q4" s="9"/>
@@ -6552,25 +6587,25 @@
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B5" s="18"/>
-      <c r="C5" s="84">
+      <c r="C5" s="79">
         <v>34.700000000000003</v>
       </c>
-      <c r="D5" s="85"/>
-      <c r="E5" s="84"/>
-      <c r="F5" s="85"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="79"/>
+      <c r="F5" s="80"/>
       <c r="G5" s="19">
         <v>5.3</v>
       </c>
       <c r="H5" s="20"/>
       <c r="I5" s="19"/>
       <c r="J5" s="19"/>
-      <c r="K5" s="84"/>
-      <c r="L5" s="85"/>
-      <c r="M5" s="84"/>
-      <c r="N5" s="85"/>
+      <c r="K5" s="79"/>
+      <c r="L5" s="80"/>
+      <c r="M5" s="79"/>
+      <c r="N5" s="80"/>
       <c r="O5" s="21">
         <f>SUM(C5:N5)</f>
         <v>40</v>
@@ -6590,19 +6625,19 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" s="25" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B6" s="25"/>
-      <c r="C6" s="86">
+      <c r="C6" s="81">
         <f>C5/$O$5</f>
         <v>0.86750000000000005</v>
       </c>
-      <c r="D6" s="87"/>
-      <c r="E6" s="86">
+      <c r="D6" s="82"/>
+      <c r="E6" s="81">
         <f>E5/$O$5</f>
         <v>0</v>
       </c>
-      <c r="F6" s="87"/>
+      <c r="F6" s="82"/>
       <c r="G6" s="26">
         <f>G5/$O$5</f>
         <v>0.13250000000000001</v>
@@ -6619,16 +6654,16 @@
         <f>J5/$O$5</f>
         <v>0</v>
       </c>
-      <c r="K6" s="86">
+      <c r="K6" s="81">
         <f>K5/$O$5</f>
         <v>0</v>
       </c>
-      <c r="L6" s="87"/>
-      <c r="M6" s="86">
+      <c r="L6" s="82"/>
+      <c r="M6" s="81">
         <f>M5/$O$5</f>
         <v>0</v>
       </c>
-      <c r="N6" s="87"/>
+      <c r="N6" s="82"/>
       <c r="O6" s="27">
         <f>SUM(C6:N6)</f>
         <v>1</v>
@@ -6648,44 +6683,44 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" s="29" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B7" s="29"/>
       <c r="C7" s="30" t="s">
+        <v>403</v>
+      </c>
+      <c r="D7" s="30" t="s">
+        <v>404</v>
+      </c>
+      <c r="E7" s="30" t="s">
+        <v>403</v>
+      </c>
+      <c r="F7" s="30" t="s">
+        <v>404</v>
+      </c>
+      <c r="G7" s="30" t="s">
         <v>405</v>
       </c>
-      <c r="D7" s="30" t="s">
-        <v>406</v>
-      </c>
-      <c r="E7" s="30" t="s">
+      <c r="H7" s="30" t="s">
         <v>405</v>
       </c>
-      <c r="F7" s="30" t="s">
-        <v>406</v>
-      </c>
-      <c r="G7" s="30" t="s">
-        <v>407</v>
-      </c>
-      <c r="H7" s="30" t="s">
-        <v>407</v>
-      </c>
       <c r="I7" s="30" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="J7" s="30" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="K7" s="30" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="L7" s="30" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="M7" s="30" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N7" s="30" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="O7" s="9"/>
       <c r="P7" s="9"/>
@@ -6703,7 +6738,7 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" s="29" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B8" s="29"/>
       <c r="C8" s="32">
@@ -6801,7 +6836,7 @@
         <v>0</v>
       </c>
       <c r="B10" s="32" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C10" s="32">
         <v>1</v>
@@ -6883,7 +6918,7 @@
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="B12" s="32"/>
       <c r="C12" s="37"/>
@@ -6958,7 +6993,7 @@
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" s="29" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B14" s="32"/>
       <c r="C14" s="37"/>
@@ -7031,10 +7066,10 @@
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" s="29" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="B16" s="32" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C16" s="37">
         <v>7.0000000000000001E-3</v>
@@ -7066,7 +7101,7 @@
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A17" s="29" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B17" s="32"/>
       <c r="C17" s="37"/>
@@ -7097,7 +7132,7 @@
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A18" s="29" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B18" s="32"/>
       <c r="C18" s="37"/>
@@ -7128,7 +7163,7 @@
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A19" s="29" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B19" s="32"/>
       <c r="C19" s="37"/>
@@ -7159,7 +7194,7 @@
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A20" s="29" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="B20" s="32"/>
       <c r="C20" s="37"/>
@@ -7221,13 +7256,13 @@
       <c r="A22" s="41"/>
       <c r="B22" s="42"/>
       <c r="C22" s="43" t="s">
+        <v>414</v>
+      </c>
+      <c r="D22" s="43" t="s">
+        <v>415</v>
+      </c>
+      <c r="E22" s="44" t="s">
         <v>416</v>
-      </c>
-      <c r="D22" s="43" t="s">
-        <v>417</v>
-      </c>
-      <c r="E22" s="44" t="s">
-        <v>418</v>
       </c>
       <c r="F22" s="45"/>
       <c r="G22" s="45"/>
@@ -7254,10 +7289,10 @@
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A23" s="29" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B23" s="32" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C23" s="35">
         <f>_xlfn.XLOOKUP(B23,Surfactant[Surfactant],Surfactant[Surf_conc.])</f>
@@ -7295,7 +7330,7 @@
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A24" s="29" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="B24" s="32"/>
       <c r="C24" s="35" t="e">
@@ -7332,7 +7367,7 @@
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A25" s="29" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="B25" s="32"/>
       <c r="C25" s="35" t="e">
@@ -7401,76 +7436,76 @@
         <v>0</v>
       </c>
       <c r="B27" s="48" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C27" s="48" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="D27" s="48" t="s">
         <v>1</v>
       </c>
       <c r="E27" s="48" t="s">
+        <v>409</v>
+      </c>
+      <c r="F27" s="48" t="s">
+        <v>410</v>
+      </c>
+      <c r="G27" s="48" t="s">
         <v>411</v>
       </c>
-      <c r="F27" s="48" t="s">
+      <c r="H27" s="48" t="s">
         <v>412</v>
       </c>
-      <c r="G27" s="48" t="s">
+      <c r="I27" s="48" t="s">
         <v>413</v>
       </c>
-      <c r="H27" s="48" t="s">
-        <v>414</v>
-      </c>
-      <c r="I27" s="48" t="s">
-        <v>415</v>
-      </c>
       <c r="J27" s="48" t="s">
+        <v>417</v>
+      </c>
+      <c r="K27" s="48" t="s">
+        <v>418</v>
+      </c>
+      <c r="L27" s="48" t="s">
         <v>419</v>
-      </c>
-      <c r="K27" s="48" t="s">
-        <v>420</v>
-      </c>
-      <c r="L27" s="48" t="s">
-        <v>421</v>
       </c>
       <c r="M27" s="48" t="s">
         <v>0</v>
       </c>
       <c r="N27" s="48" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="O27" s="48" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="P27" s="48" t="s">
         <v>1</v>
       </c>
       <c r="Q27" s="48" t="s">
+        <v>409</v>
+      </c>
+      <c r="R27" s="48" t="s">
+        <v>410</v>
+      </c>
+      <c r="S27" s="48" t="s">
         <v>411</v>
       </c>
-      <c r="R27" s="48" t="s">
+      <c r="T27" s="48" t="s">
         <v>412</v>
       </c>
-      <c r="S27" s="48" t="s">
+      <c r="U27" s="48" t="s">
         <v>413</v>
       </c>
-      <c r="T27" s="48" t="s">
-        <v>414</v>
-      </c>
-      <c r="U27" s="48" t="s">
+      <c r="V27" s="48" t="s">
+        <v>417</v>
+      </c>
+      <c r="W27" s="48" t="s">
+        <v>418</v>
+      </c>
+      <c r="X27" s="48" t="s">
+        <v>419</v>
+      </c>
+      <c r="Y27" s="48" t="s">
         <v>415</v>
-      </c>
-      <c r="V27" s="48" t="s">
-        <v>419</v>
-      </c>
-      <c r="W27" s="48" t="s">
-        <v>420</v>
-      </c>
-      <c r="X27" s="48" t="s">
-        <v>421</v>
-      </c>
-      <c r="Y27" s="48" t="s">
-        <v>417</v>
       </c>
       <c r="Z27" s="22"/>
       <c r="AA27" s="22"/>
@@ -7628,6 +7663,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="K5:L5"/>
@@ -7636,14 +7679,6 @@
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="K6:L6"/>
     <mergeCell ref="M6:N6"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <conditionalFormatting sqref="A29">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="notEqual">
@@ -7674,14 +7709,15 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x14">
       <controls>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="2049" r:id="rId3" name="Button 1">
+            <control shapeId="2049" r:id="rId4" name="Button 1">
               <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0">
                 <anchor moveWithCells="1" sizeWithCells="1">
                   <from>
@@ -7742,22 +7778,22 @@
     <col min="26" max="16384" width="6.5546875" style="73"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:25" s="62" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:25" s="62" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="B2" s="60" t="s">
+        <v>450</v>
+      </c>
+      <c r="C2" s="60" t="s">
+        <v>451</v>
+      </c>
+      <c r="D2" s="60" t="s">
         <v>452</v>
       </c>
-      <c r="C2" s="60" t="s">
-        <v>453</v>
-      </c>
-      <c r="D2" s="60" t="s">
-        <v>454</v>
-      </c>
       <c r="E2" s="60" t="s">
-        <v>455</v>
+        <v>535</v>
       </c>
       <c r="F2" s="61"/>
       <c r="G2" s="74" t="s">
-        <v>456</v>
+        <v>534</v>
       </c>
       <c r="H2" s="75"/>
       <c r="I2" s="75"/>
@@ -7765,37 +7801,37 @@
       <c r="K2" s="75"/>
       <c r="L2" s="76"/>
       <c r="M2" s="60" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
       <c r="N2" s="60" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="O2" s="74" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="P2" s="76"/>
       <c r="Q2" s="74" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="R2" s="76"/>
       <c r="S2" s="74" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="T2" s="76"/>
       <c r="U2" s="60" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="V2" s="60" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="W2" s="60" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="X2" s="60" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="Y2" s="60" t="s">
-        <v>466</v>
+        <v>533</v>
       </c>
     </row>
     <row r="3" spans="2:25" s="62" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
@@ -7804,64 +7840,64 @@
       <c r="D3" s="60"/>
       <c r="E3" s="60"/>
       <c r="F3" s="60" t="s">
+        <v>462</v>
+      </c>
+      <c r="G3" s="60" t="s">
+        <v>463</v>
+      </c>
+      <c r="H3" s="60" t="s">
+        <v>464</v>
+      </c>
+      <c r="I3" s="60" t="s">
+        <v>465</v>
+      </c>
+      <c r="J3" s="60" t="s">
+        <v>466</v>
+      </c>
+      <c r="K3" s="60" t="s">
         <v>467</v>
       </c>
-      <c r="G3" s="60" t="s">
+      <c r="L3" s="60" t="s">
         <v>468</v>
       </c>
-      <c r="H3" s="60" t="s">
+      <c r="M3" s="60" t="s">
         <v>469</v>
       </c>
-      <c r="I3" s="60" t="s">
-        <v>470</v>
-      </c>
-      <c r="J3" s="60" t="s">
-        <v>471</v>
-      </c>
-      <c r="K3" s="60" t="s">
-        <v>472</v>
-      </c>
-      <c r="L3" s="60" t="s">
-        <v>473</v>
-      </c>
-      <c r="M3" s="60" t="s">
-        <v>474</v>
-      </c>
       <c r="N3" s="60" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="O3" s="60" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P3" s="60" t="s">
         <v>14</v>
       </c>
       <c r="Q3" s="60" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="R3" s="60" t="s">
         <v>14</v>
       </c>
       <c r="S3" s="60" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T3" s="60" t="s">
         <v>14</v>
       </c>
       <c r="U3" s="60" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="V3" s="60" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="W3" s="60" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="X3" s="60" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="Y3" s="60" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
     </row>
     <row r="4" spans="2:25" s="62" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
@@ -7878,7 +7914,7 @@
         <v>3.55</v>
       </c>
       <c r="F4" s="63" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="G4" s="64"/>
       <c r="H4" s="64"/>
@@ -7887,10 +7923,10 @@
       <c r="K4" s="64"/>
       <c r="L4" s="64"/>
       <c r="M4" s="63" t="s">
-        <v>476</v>
+        <v>471</v>
       </c>
       <c r="N4" s="63" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="O4" s="63">
         <v>71</v>
@@ -7911,7 +7947,7 @@
         <v>24</v>
       </c>
       <c r="Y4" s="63" t="s">
-        <v>478</v>
+        <v>473</v>
       </c>
     </row>
     <row r="5" spans="2:25" s="62" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
@@ -7919,7 +7955,7 @@
         <v>34</v>
       </c>
       <c r="C5" s="63" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D5" s="63">
         <v>3.3</v>
@@ -7928,21 +7964,21 @@
         <v>3.6</v>
       </c>
       <c r="F5" s="63" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="G5" s="64"/>
       <c r="H5" s="64"/>
       <c r="I5" s="63" t="s">
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="J5" s="64"/>
       <c r="K5" s="64"/>
       <c r="L5" s="64"/>
       <c r="M5" s="63" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="N5" s="63" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
       <c r="O5" s="63">
         <v>97</v>
@@ -7969,15 +8005,15 @@
         <v>40</v>
       </c>
       <c r="Y5" s="65" t="s">
-        <v>483</v>
+        <v>478</v>
       </c>
     </row>
     <row r="6" spans="2:25" s="62" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
       <c r="B6" s="63" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C6" s="63" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D6" s="63">
         <v>3.5</v>
@@ -7986,23 +8022,23 @@
         <v>3.8</v>
       </c>
       <c r="F6" s="63" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="G6" s="63" t="s">
-        <v>485</v>
+        <v>480</v>
       </c>
       <c r="H6" s="64"/>
       <c r="I6" s="63" t="s">
-        <v>486</v>
+        <v>481</v>
       </c>
       <c r="J6" s="64"/>
       <c r="K6" s="64"/>
       <c r="L6" s="64"/>
       <c r="M6" s="63" t="s">
-        <v>487</v>
+        <v>482</v>
       </c>
       <c r="N6" s="63" t="s">
-        <v>488</v>
+        <v>483</v>
       </c>
       <c r="O6" s="63">
         <v>135</v>
@@ -8029,15 +8065,15 @@
         <v>38</v>
       </c>
       <c r="Y6" s="63" t="s">
-        <v>489</v>
+        <v>484</v>
       </c>
     </row>
     <row r="7" spans="2:25" s="62" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
       <c r="B7" s="60" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C7" s="60" t="s">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="D7" s="66">
         <v>3.5</v>
@@ -8046,25 +8082,25 @@
         <v>3.8</v>
       </c>
       <c r="F7" s="66" t="s">
-        <v>491</v>
+        <v>486</v>
       </c>
       <c r="G7" s="67"/>
       <c r="H7" s="67"/>
       <c r="I7" s="66" t="s">
-        <v>492</v>
+        <v>487</v>
       </c>
       <c r="J7" s="67"/>
       <c r="K7" s="66" t="s">
-        <v>493</v>
+        <v>488</v>
       </c>
       <c r="L7" s="66" t="s">
-        <v>494</v>
+        <v>489</v>
       </c>
       <c r="M7" s="66" t="s">
-        <v>495</v>
+        <v>490</v>
       </c>
       <c r="N7" s="66" t="s">
-        <v>496</v>
+        <v>491</v>
       </c>
       <c r="O7" s="66">
         <v>135</v>
@@ -8102,10 +8138,10 @@
     </row>
     <row r="8" spans="2:25" s="62" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
       <c r="B8" s="60" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C8" s="60" t="s">
-        <v>497</v>
+        <v>492</v>
       </c>
       <c r="D8" s="66">
         <v>3.5</v>
@@ -8114,25 +8150,25 @@
         <v>3.8</v>
       </c>
       <c r="F8" s="66" t="s">
-        <v>498</v>
+        <v>493</v>
       </c>
       <c r="G8" s="66" t="s">
-        <v>499</v>
+        <v>494</v>
       </c>
       <c r="H8" s="67"/>
       <c r="I8" s="67"/>
       <c r="J8" s="67"/>
       <c r="K8" s="66" t="s">
-        <v>500</v>
+        <v>495</v>
       </c>
       <c r="L8" s="66" t="s">
-        <v>501</v>
+        <v>496</v>
       </c>
       <c r="M8" s="66" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="N8" s="66" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="O8" s="66">
         <v>140</v>
@@ -8164,10 +8200,10 @@
     </row>
     <row r="9" spans="2:25" s="62" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="B9" s="60" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C9" s="60" t="s">
-        <v>497</v>
+        <v>492</v>
       </c>
       <c r="D9" s="66">
         <v>4.5</v>
@@ -8176,23 +8212,23 @@
         <v>4.8</v>
       </c>
       <c r="F9" s="66" t="s">
-        <v>504</v>
+        <v>499</v>
       </c>
       <c r="G9" s="66" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="H9" s="66" t="s">
-        <v>506</v>
+        <v>501</v>
       </c>
       <c r="I9" s="67"/>
       <c r="J9" s="67"/>
       <c r="K9" s="67"/>
       <c r="L9" s="67"/>
       <c r="M9" s="66" t="s">
-        <v>507</v>
+        <v>502</v>
       </c>
       <c r="N9" s="66" t="s">
-        <v>508</v>
+        <v>503</v>
       </c>
       <c r="O9" s="66">
         <v>160</v>
@@ -8218,10 +8254,10 @@
     </row>
     <row r="10" spans="2:25" s="62" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="B10" s="60" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C10" s="60" t="s">
-        <v>509</v>
+        <v>504</v>
       </c>
       <c r="D10" s="66">
         <v>3.5</v>
@@ -8230,25 +8266,25 @@
         <v>3.8</v>
       </c>
       <c r="F10" s="66" t="s">
-        <v>510</v>
+        <v>505</v>
       </c>
       <c r="G10" s="66" t="s">
-        <v>511</v>
+        <v>506</v>
       </c>
       <c r="H10" s="67"/>
       <c r="I10" s="66" t="s">
-        <v>512</v>
+        <v>507</v>
       </c>
       <c r="J10" s="66" t="s">
-        <v>513</v>
+        <v>508</v>
       </c>
       <c r="K10" s="67"/>
       <c r="L10" s="67"/>
       <c r="M10" s="66" t="s">
-        <v>514</v>
+        <v>509</v>
       </c>
       <c r="N10" s="68" t="s">
-        <v>515</v>
+        <v>510</v>
       </c>
       <c r="O10" s="66">
         <v>130</v>
@@ -8272,7 +8308,7 @@
         <v>70</v>
       </c>
       <c r="X10" s="66" t="s">
-        <v>516</v>
+        <v>511</v>
       </c>
       <c r="Y10" s="66">
         <v>55</v>
@@ -8280,10 +8316,10 @@
     </row>
     <row r="11" spans="2:25" s="62" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="B11" s="60" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C11" s="60" t="s">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="D11" s="66">
         <v>4.7</v>
@@ -8292,25 +8328,25 @@
         <v>5</v>
       </c>
       <c r="F11" s="66" t="s">
-        <v>517</v>
+        <v>512</v>
       </c>
       <c r="G11" s="67"/>
       <c r="H11" s="67"/>
       <c r="I11" s="66" t="s">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="J11" s="67"/>
       <c r="K11" s="66" t="s">
-        <v>519</v>
+        <v>514</v>
       </c>
       <c r="L11" s="66" t="s">
-        <v>520</v>
+        <v>515</v>
       </c>
       <c r="M11" s="66" t="s">
-        <v>514</v>
+        <v>509</v>
       </c>
       <c r="N11" s="68" t="s">
-        <v>521</v>
+        <v>516</v>
       </c>
       <c r="O11" s="66">
         <v>130</v>
@@ -8348,10 +8384,10 @@
     </row>
     <row r="12" spans="2:25" s="62" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
       <c r="B12" s="60" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C12" s="60" t="s">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="D12" s="66">
         <v>4.5</v>
@@ -8360,23 +8396,23 @@
         <v>4.8</v>
       </c>
       <c r="F12" s="66" t="s">
-        <v>522</v>
+        <v>517</v>
       </c>
       <c r="G12" s="67"/>
       <c r="H12" s="66" t="s">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="I12" s="66" t="s">
-        <v>524</v>
+        <v>519</v>
       </c>
       <c r="J12" s="67"/>
       <c r="K12" s="67"/>
       <c r="L12" s="67"/>
       <c r="M12" s="66" t="s">
-        <v>514</v>
+        <v>509</v>
       </c>
       <c r="N12" s="68" t="s">
-        <v>515</v>
+        <v>510</v>
       </c>
       <c r="O12" s="66">
         <v>130</v>
@@ -8408,10 +8444,10 @@
     </row>
     <row r="13" spans="2:25" s="62" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
       <c r="B13" s="60" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C13" s="60" t="s">
-        <v>525</v>
+        <v>520</v>
       </c>
       <c r="D13" s="66">
         <v>2.9</v>
@@ -8420,23 +8456,23 @@
         <v>3.2</v>
       </c>
       <c r="F13" s="66" t="s">
-        <v>526</v>
+        <v>521</v>
       </c>
       <c r="G13" s="67"/>
       <c r="H13" s="67"/>
       <c r="I13" s="66" t="s">
-        <v>527</v>
+        <v>522</v>
       </c>
       <c r="J13" s="67"/>
       <c r="K13" s="66" t="s">
-        <v>528</v>
+        <v>523</v>
       </c>
       <c r="L13" s="67"/>
       <c r="M13" s="66" t="s">
-        <v>529</v>
+        <v>524</v>
       </c>
       <c r="N13" s="68" t="s">
-        <v>530</v>
+        <v>525</v>
       </c>
       <c r="O13" s="66">
         <v>120</v>
@@ -8474,10 +8510,10 @@
     </row>
     <row r="14" spans="2:25" s="72" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="B14" s="60" t="s">
-        <v>537</v>
+        <v>532</v>
       </c>
       <c r="C14" s="69" t="s">
-        <v>525</v>
+        <v>520</v>
       </c>
       <c r="D14" s="70">
         <v>2.7</v>
@@ -8491,16 +8527,16 @@
       <c r="G14" s="70"/>
       <c r="H14" s="70"/>
       <c r="I14" s="70" t="s">
-        <v>531</v>
+        <v>526</v>
       </c>
       <c r="J14" s="70"/>
       <c r="K14" s="70"/>
       <c r="L14" s="70"/>
       <c r="M14" s="66" t="s">
-        <v>532</v>
+        <v>527</v>
       </c>
       <c r="N14" s="71" t="s">
-        <v>533</v>
+        <v>528</v>
       </c>
       <c r="O14" s="70">
         <v>144</v>
@@ -8518,7 +8554,7 @@
         <v>270</v>
       </c>
       <c r="T14" s="66" t="s">
-        <v>534</v>
+        <v>529</v>
       </c>
       <c r="U14" s="70">
         <v>15</v>
@@ -8537,25 +8573,25 @@
       </c>
     </row>
     <row r="15" spans="2:25" s="62" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="88" t="s">
-        <v>535</v>
-      </c>
-      <c r="C15" s="88"/>
-      <c r="D15" s="88"/>
-      <c r="E15" s="88"/>
-      <c r="F15" s="88"/>
-      <c r="G15" s="88"/>
-      <c r="H15" s="88"/>
-      <c r="I15" s="88"/>
-      <c r="J15" s="88"/>
-      <c r="K15" s="88"/>
-      <c r="L15" s="88"/>
-      <c r="M15" s="88"/>
-      <c r="N15" s="88"/>
+      <c r="B15" s="78" t="s">
+        <v>530</v>
+      </c>
+      <c r="C15" s="78"/>
+      <c r="D15" s="78"/>
+      <c r="E15" s="78"/>
+      <c r="F15" s="78"/>
+      <c r="G15" s="78"/>
+      <c r="H15" s="78"/>
+      <c r="I15" s="78"/>
+      <c r="J15" s="78"/>
+      <c r="K15" s="78"/>
+      <c r="L15" s="78"/>
+      <c r="M15" s="78"/>
+      <c r="N15" s="78"/>
     </row>
     <row r="16" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B16" s="77" t="s">
-        <v>536</v>
+        <v>531</v>
       </c>
       <c r="C16" s="77"/>
       <c r="D16" s="77"/>

</xml_diff>